<commit_message>
chore: guardar cambios pendientes de hoy
</commit_message>
<xml_diff>
--- a/tests/Plan test - seguimiento .xlsx
+++ b/tests/Plan test - seguimiento .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esus_\Documents\AI\ZTWQ\c2pro\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88AC26BD-E64A-464B-B8A2-C0FEF1376397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D1AF15-6B07-4FFF-A790-7B3EC293CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2070" windowWidth="23280" windowHeight="12480" tabRatio="601" activeTab="1" xr2:uid="{297FDD56-996B-4A91-B117-D5E5BF79AC61}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="601" activeTab="1" xr2:uid="{297FDD56-996B-4A91-B117-D5E5BF79AC61}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -2295,10 +2295,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
@@ -2340,9 +2340,13 @@
       <sheetName val="promt"/>
       <sheetName val="plan test"/>
       <sheetName val="lista frontend"/>
+      <sheetName val="Hoja1"/>
       <sheetName val="Prmot frontend"/>
       <sheetName val="lista IA "/>
       <sheetName val="prmot llm"/>
+      <sheetName val="Hoja3"/>
+      <sheetName val="FrontEND 2"/>
+      <sheetName val="LangGraph"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -11052,6 +11056,10 @@
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
       <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -11375,22 +11383,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F10C4-C2EB-41C2-BD87-B191B0E5D966}">
   <dimension ref="A1:Q404"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="29.140625" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="29.109375" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="17.6640625" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
     <col min="7" max="8" width="0" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="39.5703125" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="39.5703125" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.5546875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="39.5546875" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16.5" thickBot="1">
+    <row r="1" spans="1:11" ht="16.2" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11421,7 +11429,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="31.5" thickBot="1">
+    <row r="2" spans="1:11" ht="31.2" thickBot="1">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -11452,7 +11460,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="31.5" thickBot="1">
+    <row r="3" spans="1:11" ht="31.2" thickBot="1">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -11480,7 +11488,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="31.5" thickBot="1">
+    <row r="4" spans="1:11" ht="31.2" thickBot="1">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -11508,7 +11516,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="46.5" thickBot="1">
+    <row r="5" spans="1:11" ht="46.2" thickBot="1">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -11536,7 +11544,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="31.5" thickBot="1">
+    <row r="6" spans="1:11" ht="31.2" thickBot="1">
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
@@ -11564,7 +11572,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="31.5" thickBot="1">
+    <row r="7" spans="1:11" ht="31.2" thickBot="1">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
@@ -11592,7 +11600,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="31.5" thickBot="1">
+    <row r="8" spans="1:11" ht="31.2" thickBot="1">
       <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
@@ -11620,7 +11628,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="31.5" thickBot="1">
+    <row r="9" spans="1:11" ht="31.2" thickBot="1">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -11648,7 +11656,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="31.5" thickBot="1">
+    <row r="10" spans="1:11" ht="31.2" thickBot="1">
       <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
@@ -11676,7 +11684,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="31.5" thickBot="1">
+    <row r="11" spans="1:11" ht="31.2" thickBot="1">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
@@ -11704,7 +11712,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="31.5" thickBot="1">
+    <row r="12" spans="1:11" ht="31.2" thickBot="1">
       <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
@@ -11732,7 +11740,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="31.5" thickBot="1">
+    <row r="13" spans="1:11" ht="31.2" thickBot="1">
       <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
@@ -11760,7 +11768,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="31.5" thickBot="1">
+    <row r="14" spans="1:11" ht="31.2" thickBot="1">
       <c r="A14" s="4" t="s">
         <v>8</v>
       </c>
@@ -11788,7 +11796,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="31.5" thickBot="1">
+    <row r="15" spans="1:11" ht="31.2" thickBot="1">
       <c r="A15" s="4" t="s">
         <v>8</v>
       </c>
@@ -11816,7 +11824,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="31.5" thickBot="1">
+    <row r="16" spans="1:11" ht="31.2" thickBot="1">
       <c r="A16" s="4" t="s">
         <v>8</v>
       </c>
@@ -11844,7 +11852,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="31.5" thickBot="1">
+    <row r="17" spans="1:17" ht="31.2" thickBot="1">
       <c r="A17" s="4" t="s">
         <v>8</v>
       </c>
@@ -11872,7 +11880,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="46.5" thickBot="1">
+    <row r="18" spans="1:17" ht="31.2" thickBot="1">
       <c r="A18" s="4" t="s">
         <v>8</v>
       </c>
@@ -11900,7 +11908,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="31.5" thickBot="1">
+    <row r="19" spans="1:17" ht="31.2" thickBot="1">
       <c r="A19" s="4" t="s">
         <v>8</v>
       </c>
@@ -11928,7 +11936,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="31.5" thickBot="1">
+    <row r="20" spans="1:17" ht="31.2" thickBot="1">
       <c r="A20" s="4" t="s">
         <v>8</v>
       </c>
@@ -11956,7 +11964,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="31.5" thickBot="1">
+    <row r="21" spans="1:17" ht="31.2" thickBot="1">
       <c r="A21" s="4" t="s">
         <v>8</v>
       </c>
@@ -11984,7 +11992,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="31.5" thickBot="1">
+    <row r="22" spans="1:17" ht="31.2" thickBot="1">
       <c r="A22" s="4" t="s">
         <v>8</v>
       </c>
@@ -12012,7 +12020,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="31.5" thickBot="1">
+    <row r="23" spans="1:17" ht="31.2" thickBot="1">
       <c r="A23" s="4" t="s">
         <v>8</v>
       </c>
@@ -12040,7 +12048,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="31.5" thickBot="1">
+    <row r="24" spans="1:17" ht="31.2" thickBot="1">
       <c r="A24" s="4" t="s">
         <v>37</v>
       </c>
@@ -12075,7 +12083,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="31.5" thickBot="1">
+    <row r="25" spans="1:17" ht="31.2" thickBot="1">
       <c r="A25" s="4" t="s">
         <v>37</v>
       </c>
@@ -12110,7 +12118,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="31.5" thickBot="1">
+    <row r="26" spans="1:17" ht="31.2" thickBot="1">
       <c r="A26" s="4" t="s">
         <v>37</v>
       </c>
@@ -12145,7 +12153,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="31.5" thickBot="1">
+    <row r="27" spans="1:17" ht="31.2" thickBot="1">
       <c r="A27" s="4" t="s">
         <v>37</v>
       </c>
@@ -12180,7 +12188,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="31.5" thickBot="1">
+    <row r="28" spans="1:17" ht="31.2" thickBot="1">
       <c r="A28" s="4" t="s">
         <v>37</v>
       </c>
@@ -12215,7 +12223,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="31.5" thickBot="1">
+    <row r="29" spans="1:17" ht="31.2" thickBot="1">
       <c r="A29" s="4" t="s">
         <v>37</v>
       </c>
@@ -12250,7 +12258,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="31.5" thickBot="1">
+    <row r="30" spans="1:17" ht="31.2" thickBot="1">
       <c r="A30" s="4" t="s">
         <v>37</v>
       </c>
@@ -12285,7 +12293,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="31.5" thickBot="1">
+    <row r="31" spans="1:17" ht="31.2" thickBot="1">
       <c r="A31" s="4" t="s">
         <v>37</v>
       </c>
@@ -12320,7 +12328,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="31.5" thickBot="1">
+    <row r="32" spans="1:17" ht="31.2" thickBot="1">
       <c r="A32" s="4" t="s">
         <v>37</v>
       </c>
@@ -12355,7 +12363,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="31.5" thickBot="1">
+    <row r="33" spans="1:17" ht="31.2" thickBot="1">
       <c r="A33" s="4" t="s">
         <v>37</v>
       </c>
@@ -12390,7 +12398,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="31.5" thickBot="1">
+    <row r="34" spans="1:17" ht="31.2" thickBot="1">
       <c r="A34" s="4" t="s">
         <v>37</v>
       </c>
@@ -12425,7 +12433,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="31.5" thickBot="1">
+    <row r="35" spans="1:17" ht="31.2" thickBot="1">
       <c r="A35" s="4" t="s">
         <v>37</v>
       </c>
@@ -12460,7 +12468,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="31.5" thickBot="1">
+    <row r="36" spans="1:17" ht="31.2" thickBot="1">
       <c r="A36" s="4" t="s">
         <v>37</v>
       </c>
@@ -12495,7 +12503,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="31.5" thickBot="1">
+    <row r="37" spans="1:17" ht="31.2" thickBot="1">
       <c r="A37" s="4" t="s">
         <v>37</v>
       </c>
@@ -12530,7 +12538,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="31.5" thickBot="1">
+    <row r="38" spans="1:17" ht="31.2" thickBot="1">
       <c r="A38" s="4" t="s">
         <v>37</v>
       </c>
@@ -12565,7 +12573,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="31.5" thickBot="1">
+    <row r="39" spans="1:17" ht="31.2" thickBot="1">
       <c r="A39" s="4" t="s">
         <v>37</v>
       </c>
@@ -12600,7 +12608,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="31.5" thickBot="1">
+    <row r="40" spans="1:17" ht="31.2" thickBot="1">
       <c r="A40" s="4" t="s">
         <v>37</v>
       </c>
@@ -12635,7 +12643,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="31.5" thickBot="1">
+    <row r="41" spans="1:17" ht="31.2" thickBot="1">
       <c r="A41" s="4" t="s">
         <v>73</v>
       </c>
@@ -12667,7 +12675,7 @@
         <v>TS-UC-SEC-MCP-003test_001_query_under_5s_allowed</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="31.5" thickBot="1">
+    <row r="42" spans="1:17" ht="31.2" thickBot="1">
       <c r="A42" s="4" t="s">
         <v>73</v>
       </c>
@@ -12699,7 +12707,7 @@
         <v>TS-UC-SEC-MCP-003test_002_query_at_5s_allowed</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="31.5" thickBot="1">
+    <row r="43" spans="1:17" ht="31.2" thickBot="1">
       <c r="A43" s="4" t="s">
         <v>73</v>
       </c>
@@ -12731,7 +12739,7 @@
         <v>TS-UC-SEC-MCP-003test_003_query_over_5s_timeout_cancelled</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="31.5" thickBot="1">
+    <row r="44" spans="1:17" ht="31.2" thickBot="1">
       <c r="A44" s="4" t="s">
         <v>73</v>
       </c>
@@ -12763,7 +12771,7 @@
         <v>TS-UC-SEC-MCP-003test_004_query_result_under_1000_rows_allowed</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="31.5" thickBot="1">
+    <row r="45" spans="1:17" ht="31.2" thickBot="1">
       <c r="A45" s="4" t="s">
         <v>73</v>
       </c>
@@ -12795,7 +12803,7 @@
         <v>TS-UC-SEC-MCP-003test_005_query_result_at_1000_rows_allowed</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="31.5" thickBot="1">
+    <row r="46" spans="1:17" ht="31.2" thickBot="1">
       <c r="A46" s="4" t="s">
         <v>73</v>
       </c>
@@ -12827,7 +12835,7 @@
         <v>TS-UC-SEC-MCP-003test_006_query_result_over_1000_rows_truncated</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="31.5" thickBot="1">
+    <row r="47" spans="1:17" ht="31.2" thickBot="1">
       <c r="A47" s="4" t="s">
         <v>73</v>
       </c>
@@ -12859,7 +12867,7 @@
         <v>TS-UC-SEC-MCP-003test_007_query_result_truncated_flag_set</v>
       </c>
     </row>
-    <row r="48" spans="1:17" ht="31.5" thickBot="1">
+    <row r="48" spans="1:17" ht="31.2" thickBot="1">
       <c r="A48" s="4" t="s">
         <v>73</v>
       </c>
@@ -12891,7 +12899,7 @@
         <v>TS-UC-SEC-MCP-003test_008_timeout_returns_partial_results</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="31.5" thickBot="1">
+    <row r="49" spans="1:11" ht="31.2" thickBot="1">
       <c r="A49" s="4" t="s">
         <v>73</v>
       </c>
@@ -12923,7 +12931,7 @@
         <v>TS-UC-SEC-MCP-003test_009_timeout_audit_log_created</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="31.5" thickBot="1">
+    <row r="50" spans="1:11" ht="31.2" thickBot="1">
       <c r="A50" s="4" t="s">
         <v>73</v>
       </c>
@@ -12955,7 +12963,7 @@
         <v>TS-UC-SEC-MCP-003test_010_row_limit_audit_log_created</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="31.5" thickBot="1">
+    <row r="51" spans="1:11" ht="31.2" thickBot="1">
       <c r="A51" s="4" t="s">
         <v>73</v>
       </c>
@@ -12987,7 +12995,7 @@
         <v>TS-UC-SEC-MCP-003test_011_combined_timeout_and_row_limit</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="31.5" thickBot="1">
+    <row r="52" spans="1:11" ht="31.2" thickBot="1">
       <c r="A52" s="4" t="s">
         <v>73</v>
       </c>
@@ -13019,7 +13027,7 @@
         <v>TS-UC-SEC-MCP-003test_012_query_limit_config_per_tenant</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="31.5" thickBot="1">
+    <row r="53" spans="1:11" ht="31.2" thickBot="1">
       <c r="A53" s="4" t="s">
         <v>73</v>
       </c>
@@ -13051,7 +13059,7 @@
         <v>TS-UC-SEC-MCP-003test_edge_001_exactly_1000_rows</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="31.5" thickBot="1">
+    <row r="54" spans="1:11" ht="31.2" thickBot="1">
       <c r="A54" s="4" t="s">
         <v>73</v>
       </c>
@@ -13083,7 +13091,7 @@
         <v>TS-UC-SEC-MCP-003test_edge_002_empty_result_set</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="31.5" thickBot="1">
+    <row r="55" spans="1:11" ht="31.2" thickBot="1">
       <c r="A55" s="4" t="s">
         <v>73</v>
       </c>
@@ -13115,7 +13123,7 @@
         <v>TS-UC-SEC-MCP-003test_edge_003_streaming_query_timeout</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="31.5" thickBot="1">
+    <row r="56" spans="1:11" ht="31.2" thickBot="1">
       <c r="A56" s="4" t="s">
         <v>91</v>
       </c>
@@ -13147,7 +13155,7 @@
         <v>TS-UC-SEC-ANO-001test_001_detect_dni_valid_12345678Z</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="31.5" thickBot="1">
+    <row r="57" spans="1:11" ht="31.2" thickBot="1">
       <c r="A57" s="4" t="s">
         <v>91</v>
       </c>
@@ -13179,7 +13187,7 @@
         <v>TS-UC-SEC-ANO-001test_002_detect_dni_valid_87654321X</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="31.5" thickBot="1">
+    <row r="58" spans="1:11" ht="31.2" thickBot="1">
       <c r="A58" s="4" t="s">
         <v>91</v>
       </c>
@@ -13211,7 +13219,7 @@
         <v>TS-UC-SEC-ANO-001test_003_detect_dni_invalid_length_9_digits</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="31.5" thickBot="1">
+    <row r="59" spans="1:11" ht="31.2" thickBot="1">
       <c r="A59" s="4" t="s">
         <v>91</v>
       </c>
@@ -13243,7 +13251,7 @@
         <v>TS-UC-SEC-ANO-001test_004_detect_dni_invalid_length_7_digits</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="31.5" thickBot="1">
+    <row r="60" spans="1:11" ht="31.2" thickBot="1">
       <c r="A60" s="4" t="s">
         <v>91</v>
       </c>
@@ -13275,7 +13283,7 @@
         <v>TS-UC-SEC-ANO-001test_005_detect_dni_invalid_letter_checksum</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="31.5" thickBot="1">
+    <row r="61" spans="1:11" ht="31.2" thickBot="1">
       <c r="A61" s="4" t="s">
         <v>91</v>
       </c>
@@ -13307,7 +13315,7 @@
         <v>TS-UC-SEC-ANO-001test_006_detect_multiple_dnis_in_text</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="31.5" thickBot="1">
+    <row r="62" spans="1:11" ht="31.2" thickBot="1">
       <c r="A62" s="4" t="s">
         <v>91</v>
       </c>
@@ -13339,7 +13347,7 @@
         <v>TS-UC-SEC-ANO-001test_007_detect_email_simple</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="31.5" thickBot="1">
+    <row r="63" spans="1:11" ht="31.2" thickBot="1">
       <c r="A63" s="4" t="s">
         <v>91</v>
       </c>
@@ -13371,7 +13379,7 @@
         <v>TS-UC-SEC-ANO-001test_008_detect_email_with_subdomain</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="31.5" thickBot="1">
+    <row r="64" spans="1:11" ht="31.2" thickBot="1">
       <c r="A64" s="4" t="s">
         <v>91</v>
       </c>
@@ -13403,7 +13411,7 @@
         <v>TS-UC-SEC-ANO-001test_009_detect_email_with_plus_sign</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="31.5" thickBot="1">
+    <row r="65" spans="1:11" ht="31.2" thickBot="1">
       <c r="A65" s="4" t="s">
         <v>91</v>
       </c>
@@ -13435,7 +13443,7 @@
         <v>TS-UC-SEC-ANO-001test_010_detect_email_invalid_no_at</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="31.5" thickBot="1">
+    <row r="66" spans="1:11" ht="31.2" thickBot="1">
       <c r="A66" s="4" t="s">
         <v>91</v>
       </c>
@@ -13467,7 +13475,7 @@
         <v>TS-UC-SEC-ANO-001test_011_detect_multiple_emails_in_text</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="31.5" thickBot="1">
+    <row r="67" spans="1:11" ht="31.2" thickBot="1">
       <c r="A67" s="4" t="s">
         <v>91</v>
       </c>
@@ -13499,7 +13507,7 @@
         <v>TS-UC-SEC-ANO-001test_012_detect_phone_mobile_612345678</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="31.5" thickBot="1">
+    <row r="68" spans="1:11" ht="31.2" thickBot="1">
       <c r="A68" s="4" t="s">
         <v>91</v>
       </c>
@@ -13531,7 +13539,7 @@
         <v>TS-UC-SEC-ANO-001test_013_detect_phone_mobile_with_prefix_34</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="31.5" thickBot="1">
+    <row r="69" spans="1:11" ht="31.2" thickBot="1">
       <c r="A69" s="4" t="s">
         <v>91</v>
       </c>
@@ -13563,7 +13571,7 @@
         <v>TS-UC-SEC-ANO-001test_014_detect_phone_landline_912345678</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="31.5" thickBot="1">
+    <row r="70" spans="1:11" ht="31.2" thickBot="1">
       <c r="A70" s="4" t="s">
         <v>91</v>
       </c>
@@ -13595,7 +13603,7 @@
         <v>TS-UC-SEC-ANO-001test_015_detect_phone_invalid_short</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="31.5" thickBot="1">
+    <row r="71" spans="1:11" ht="31.2" thickBot="1">
       <c r="A71" s="4" t="s">
         <v>91</v>
       </c>
@@ -13627,7 +13635,7 @@
         <v>TS-UC-SEC-ANO-001test_016_detect_multiple_phones_in_text</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="31.5" thickBot="1">
+    <row r="72" spans="1:11" ht="31.2" thickBot="1">
       <c r="A72" s="4" t="s">
         <v>91</v>
       </c>
@@ -13659,7 +13667,7 @@
         <v>TS-UC-SEC-ANO-001test_017_detect_iban_spain_valid</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="31.5" thickBot="1">
+    <row r="73" spans="1:11" ht="31.2" thickBot="1">
       <c r="A73" s="4" t="s">
         <v>91</v>
       </c>
@@ -13691,7 +13699,7 @@
         <v>TS-UC-SEC-ANO-001test_018_detect_iban_germany_valid</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="31.5" thickBot="1">
+    <row r="74" spans="1:11" ht="31.2" thickBot="1">
       <c r="A74" s="4" t="s">
         <v>91</v>
       </c>
@@ -13723,7 +13731,7 @@
         <v>TS-UC-SEC-ANO-001test_019_detect_iban_invalid_checksum</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="31.5" thickBot="1">
+    <row r="75" spans="1:11" ht="31.2" thickBot="1">
       <c r="A75" s="4" t="s">
         <v>91</v>
       </c>
@@ -13755,7 +13763,7 @@
         <v>TS-UC-SEC-ANO-001test_020_detect_iban_invalid_length</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="31.5" thickBot="1">
+    <row r="76" spans="1:11" ht="31.2" thickBot="1">
       <c r="A76" s="4" t="s">
         <v>91</v>
       </c>
@@ -13787,7 +13795,7 @@
         <v>TS-UC-SEC-ANO-001test_021_detect_all_pii_types_in_document</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="31.5" thickBot="1">
+    <row r="77" spans="1:11" ht="31.2" thickBot="1">
       <c r="A77" s="4" t="s">
         <v>91</v>
       </c>
@@ -13819,7 +13827,7 @@
         <v>TS-UC-SEC-ANO-001test_022_detect_no_pii_clean_document</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="31.5" thickBot="1">
+    <row r="78" spans="1:11" ht="31.2" thickBot="1">
       <c r="A78" s="4" t="s">
         <v>91</v>
       </c>
@@ -13851,7 +13859,7 @@
         <v>TS-UC-SEC-ANO-001test_023_detect_pii_positions_returned</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="31.5" thickBot="1">
+    <row r="79" spans="1:11" ht="31.2" thickBot="1">
       <c r="A79" s="4" t="s">
         <v>91</v>
       </c>
@@ -13883,7 +13891,7 @@
         <v>TS-UC-SEC-ANO-001test_024_detect_pii_counts_by_type</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="31.5" thickBot="1">
+    <row r="80" spans="1:11" ht="31.2" thickBot="1">
       <c r="A80" s="4" t="s">
         <v>91</v>
       </c>
@@ -13915,7 +13923,7 @@
         <v>TS-UC-SEC-ANO-001test_edge_001_pii_in_different_languages</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="31.5" thickBot="1">
+    <row r="81" spans="1:11" ht="31.2" thickBot="1">
       <c r="A81" s="4" t="s">
         <v>91</v>
       </c>
@@ -13947,7 +13955,7 @@
         <v>TS-UC-SEC-ANO-001test_edge_002_pii_with_unicode_characters</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="31.5" thickBot="1">
+    <row r="82" spans="1:11" ht="31.2" thickBot="1">
       <c r="A82" s="4" t="s">
         <v>91</v>
       </c>
@@ -13970,7 +13978,7 @@
         <v>TS-UC-SEC-ANO-001test_edge_003_pii_in_html_escaped_text</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="31.5" thickBot="1">
+    <row r="83" spans="1:11" ht="31.2" thickBot="1">
       <c r="A83" s="4" t="s">
         <v>120</v>
       </c>
@@ -13999,7 +14007,7 @@
         <v>TS-UC-SEC-ANO-002test_001_redact_dni_to_redacted</v>
       </c>
     </row>
-    <row r="84" spans="1:11" ht="31.5" thickBot="1">
+    <row r="84" spans="1:11" ht="31.2" thickBot="1">
       <c r="A84" s="4" t="s">
         <v>120</v>
       </c>
@@ -14028,7 +14036,7 @@
         <v>TS-UC-SEC-ANO-002test_002_redact_email_to_redacted</v>
       </c>
     </row>
-    <row r="85" spans="1:11" ht="31.5" thickBot="1">
+    <row r="85" spans="1:11" ht="31.2" thickBot="1">
       <c r="A85" s="4" t="s">
         <v>120</v>
       </c>
@@ -14057,7 +14065,7 @@
         <v>TS-UC-SEC-ANO-002test_003_redact_phone_to_redacted</v>
       </c>
     </row>
-    <row r="86" spans="1:11" ht="31.5" thickBot="1">
+    <row r="86" spans="1:11" ht="31.2" thickBot="1">
       <c r="A86" s="4" t="s">
         <v>120</v>
       </c>
@@ -14086,7 +14094,7 @@
         <v>TS-UC-SEC-ANO-002test_004_redact_multiple_pii_all_redacted</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="31.5" thickBot="1">
+    <row r="87" spans="1:11" ht="31.2" thickBot="1">
       <c r="A87" s="4" t="s">
         <v>120</v>
       </c>
@@ -14115,7 +14123,7 @@
         <v>TS-UC-SEC-ANO-002test_005_hash_dni_deterministic</v>
       </c>
     </row>
-    <row r="88" spans="1:11" ht="31.5" thickBot="1">
+    <row r="88" spans="1:11" ht="31.2" thickBot="1">
       <c r="A88" s="4" t="s">
         <v>120</v>
       </c>
@@ -14144,7 +14152,7 @@
         <v>TS-UC-SEC-ANO-002test_006_hash_same_value_same_hash</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="31.5" thickBot="1">
+    <row r="89" spans="1:11" ht="31.2" thickBot="1">
       <c r="A89" s="4" t="s">
         <v>120</v>
       </c>
@@ -14173,7 +14181,7 @@
         <v>TS-UC-SEC-ANO-002test_007_hash_different_values_different_hash</v>
       </c>
     </row>
-    <row r="90" spans="1:11" ht="31.5" thickBot="1">
+    <row r="90" spans="1:11" ht="31.2" thickBot="1">
       <c r="A90" s="4" t="s">
         <v>120</v>
       </c>
@@ -14202,7 +14210,7 @@
         <v>TS-UC-SEC-ANO-002test_008_hash_irreversible_validation</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="31.5" thickBot="1">
+    <row r="91" spans="1:11" ht="31.2" thickBot="1">
       <c r="A91" s="4" t="s">
         <v>120</v>
       </c>
@@ -14231,7 +14239,7 @@
         <v>TS-UC-SEC-ANO-002test_009_pseudonymize_name_to_persona_001</v>
       </c>
     </row>
-    <row r="92" spans="1:11" ht="31.5" thickBot="1">
+    <row r="92" spans="1:11" ht="31.2" thickBot="1">
       <c r="A92" s="4" t="s">
         <v>120</v>
       </c>
@@ -14260,7 +14268,7 @@
         <v>TS-UC-SEC-ANO-002test_010_pseudonymize_consistent_same_name</v>
       </c>
     </row>
-    <row r="93" spans="1:11" ht="46.5" thickBot="1">
+    <row r="93" spans="1:11" ht="31.2" thickBot="1">
       <c r="A93" s="4" t="s">
         <v>120</v>
       </c>
@@ -14289,7 +14297,7 @@
         <v>TS-UC-SEC-ANO-002test_011_pseudonymize_different_names_different_ids</v>
       </c>
     </row>
-    <row r="94" spans="1:11" ht="31.5" thickBot="1">
+    <row r="94" spans="1:11" ht="31.2" thickBot="1">
       <c r="A94" s="4" t="s">
         <v>120</v>
       </c>
@@ -14318,7 +14326,7 @@
         <v>TS-UC-SEC-ANO-002test_012_pseudonymize_in_context_preserved</v>
       </c>
     </row>
-    <row r="95" spans="1:11" ht="31.5" thickBot="1">
+    <row r="95" spans="1:11" ht="31.2" thickBot="1">
       <c r="A95" s="4" t="s">
         <v>120</v>
       </c>
@@ -14347,7 +14355,7 @@
         <v>TS-UC-SEC-ANO-002test_013_strategy_by_pii_type_default</v>
       </c>
     </row>
-    <row r="96" spans="1:11" ht="31.5" thickBot="1">
+    <row r="96" spans="1:11" ht="31.2" thickBot="1">
       <c r="A96" s="4" t="s">
         <v>120</v>
       </c>
@@ -14376,7 +14384,7 @@
         <v>TS-UC-SEC-ANO-002test_014_strategy_by_tenant_config</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="31.5" thickBot="1">
+    <row r="97" spans="1:11" ht="31.2" thickBot="1">
       <c r="A97" s="4" t="s">
         <v>120</v>
       </c>
@@ -14405,7 +14413,7 @@
         <v>TS-UC-SEC-ANO-002test_015_strategy_mixed_per_type</v>
       </c>
     </row>
-    <row r="98" spans="1:11" ht="31.5" thickBot="1">
+    <row r="98" spans="1:11" ht="31.2" thickBot="1">
       <c r="A98" s="4" t="s">
         <v>120</v>
       </c>
@@ -14434,7 +14442,7 @@
         <v>TS-UC-SEC-ANO-002test_016_strategy_none_keeps_original</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="31.5" thickBot="1">
+    <row r="99" spans="1:11" ht="31.2" thickBot="1">
       <c r="A99" s="4" t="s">
         <v>120</v>
       </c>
@@ -14463,7 +14471,7 @@
         <v>TS-UC-SEC-ANO-002test_edge_001_nested_pii_in_pii</v>
       </c>
     </row>
-    <row r="100" spans="1:11" ht="31.5" thickBot="1">
+    <row r="100" spans="1:11" ht="31.2" thickBot="1">
       <c r="A100" s="4" t="s">
         <v>120</v>
       </c>
@@ -14492,7 +14500,7 @@
         <v>TS-UC-SEC-ANO-002test_edge_002_overlapping_pii_positions</v>
       </c>
     </row>
-    <row r="101" spans="1:11" ht="31.5" thickBot="1">
+    <row r="101" spans="1:11" ht="31.2" thickBot="1">
       <c r="A101" s="4" t="s">
         <v>120</v>
       </c>
@@ -14521,7 +14529,7 @@
         <v>TS-UC-SEC-ANO-002test_edge_003_empty_text_no_error</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="16.5" thickBot="1">
+    <row r="102" spans="1:11" ht="16.2" thickBot="1">
       <c r="A102" s="4" t="s">
         <v>141</v>
       </c>
@@ -14550,7 +14558,7 @@
         <v>TS-UC-SEC-ANO-003Tests not individually listed</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="16.5" thickBot="1">
+    <row r="103" spans="1:11" ht="16.2" thickBot="1">
       <c r="A103" s="4" t="s">
         <v>144</v>
       </c>
@@ -14579,7 +14587,7 @@
         <v>TS-UC-SEC-TNT-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="16.5" thickBot="1">
+    <row r="104" spans="1:11" ht="16.2" thickBot="1">
       <c r="A104" s="4" t="s">
         <v>145</v>
       </c>
@@ -14605,7 +14613,7 @@
         <v>TS-UC-SEC-JWT-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="16.5" thickBot="1">
+    <row r="105" spans="1:11" ht="16.2" thickBot="1">
       <c r="A105" s="4" t="s">
         <v>146</v>
       </c>
@@ -14631,7 +14639,7 @@
         <v>TS-UC-SEC-AUD-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="31.5" thickBot="1">
+    <row r="106" spans="1:11" ht="31.2" thickBot="1">
       <c r="A106" s="4" t="s">
         <v>147</v>
       </c>
@@ -14660,7 +14668,7 @@
         <v>TS-UC-SEC-GAM-001test_001_mass_changes_11_in_hour_detected</v>
       </c>
     </row>
-    <row r="107" spans="1:11" ht="31.5" thickBot="1">
+    <row r="107" spans="1:11" ht="31.2" thickBot="1">
       <c r="A107" s="4" t="s">
         <v>147</v>
       </c>
@@ -14689,7 +14697,7 @@
         <v>TS-UC-SEC-GAM-001test_002_mass_changes_10_in_hour_allowed</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="31.5" thickBot="1">
+    <row r="108" spans="1:11" ht="31.2" thickBot="1">
       <c r="A108" s="4" t="s">
         <v>147</v>
       </c>
@@ -14718,7 +14726,7 @@
         <v>TS-UC-SEC-GAM-001test_003_mass_changes_window_reset</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="31.5" thickBot="1">
+    <row r="109" spans="1:11" ht="31.2" thickBot="1">
       <c r="A109" s="4" t="s">
         <v>147</v>
       </c>
@@ -14747,7 +14755,7 @@
         <v>TS-UC-SEC-GAM-001test_004_resolve_reintroduce_3_times_detected</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="31.5" thickBot="1">
+    <row r="110" spans="1:11" ht="31.2" thickBot="1">
       <c r="A110" s="4" t="s">
         <v>147</v>
       </c>
@@ -14776,7 +14784,7 @@
         <v>TS-UC-SEC-GAM-001test_005_resolve_reintroduce_2_times_allowed</v>
       </c>
     </row>
-    <row r="111" spans="1:11" ht="31.5" thickBot="1">
+    <row r="111" spans="1:11" ht="31.2" thickBot="1">
       <c r="A111" s="4" t="s">
         <v>147</v>
       </c>
@@ -14805,7 +14813,7 @@
         <v>TS-UC-SEC-GAM-001test_006_resolve_reintroduce_different_hash_allowed</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="31.5" thickBot="1">
+    <row r="112" spans="1:11" ht="31.2" thickBot="1">
       <c r="A112" s="4" t="s">
         <v>147</v>
       </c>
@@ -14834,7 +14842,7 @@
         <v>TS-UC-SEC-GAM-001test_007_high_score_few_docs_detected</v>
       </c>
     </row>
-    <row r="113" spans="1:11" ht="31.5" thickBot="1">
+    <row r="113" spans="1:11" ht="31.2" thickBot="1">
       <c r="A113" s="4" t="s">
         <v>147</v>
       </c>
@@ -14863,7 +14871,7 @@
         <v>TS-UC-SEC-GAM-001test_008_high_score_many_docs_allowed</v>
       </c>
     </row>
-    <row r="114" spans="1:11" ht="31.5" thickBot="1">
+    <row r="114" spans="1:11" ht="31.2" thickBot="1">
       <c r="A114" s="4" t="s">
         <v>147</v>
       </c>
@@ -14892,7 +14900,7 @@
         <v>TS-UC-SEC-GAM-001test_009_high_score_threshold_boundary</v>
       </c>
     </row>
-    <row r="115" spans="1:11" ht="31.5" thickBot="1">
+    <row r="115" spans="1:11" ht="31.2" thickBot="1">
       <c r="A115" s="4" t="s">
         <v>147</v>
       </c>
@@ -14921,7 +14929,7 @@
         <v>TS-UC-SEC-GAM-001test_010_weight_change_25_percent_detected</v>
       </c>
     </row>
-    <row r="116" spans="1:11" ht="31.5" thickBot="1">
+    <row r="116" spans="1:11" ht="31.2" thickBot="1">
       <c r="A116" s="4" t="s">
         <v>147</v>
       </c>
@@ -14950,7 +14958,7 @@
         <v>TS-UC-SEC-GAM-001test_011_weight_change_15_percent_allowed</v>
       </c>
     </row>
-    <row r="117" spans="1:11" ht="31.5" thickBot="1">
+    <row r="117" spans="1:11" ht="31.2" thickBot="1">
       <c r="A117" s="4" t="s">
         <v>147</v>
       </c>
@@ -14979,7 +14987,7 @@
         <v>TS-UC-SEC-GAM-001test_012_weight_change_tracking_24h_window</v>
       </c>
     </row>
-    <row r="118" spans="1:11" ht="31.5" thickBot="1">
+    <row r="118" spans="1:11" ht="31.2" thickBot="1">
       <c r="A118" s="4" t="s">
         <v>147</v>
       </c>
@@ -15008,7 +15016,7 @@
         <v>TS-UC-SEC-GAM-001test_edge_001_multiple_violations_combined</v>
       </c>
     </row>
-    <row r="119" spans="1:11" ht="31.5" thickBot="1">
+    <row r="119" spans="1:11" ht="31.2" thickBot="1">
       <c r="A119" s="4" t="s">
         <v>147</v>
       </c>
@@ -15037,7 +15045,7 @@
         <v>TS-UC-SEC-GAM-001test_edge_002_violation_penalty_application</v>
       </c>
     </row>
-    <row r="120" spans="1:11" ht="31.5" thickBot="1">
+    <row r="120" spans="1:11" ht="31.2" thickBot="1">
       <c r="A120" s="4" t="s">
         <v>147</v>
       </c>
@@ -15066,7 +15074,7 @@
         <v>TS-UC-SEC-GAM-001test_edge_003_violation_audit_logging</v>
       </c>
     </row>
-    <row r="121" spans="1:11" ht="31.5" thickBot="1">
+    <row r="121" spans="1:11" ht="31.2" thickBot="1">
       <c r="A121" s="4" t="s">
         <v>163</v>
       </c>
@@ -15098,7 +15106,7 @@
         <v>TS-UD-DOC-CLS-001test_001_clause_creation_with_all_fields</v>
       </c>
     </row>
-    <row r="122" spans="1:11" ht="31.5" thickBot="1">
+    <row r="122" spans="1:11" ht="31.2" thickBot="1">
       <c r="A122" s="4" t="s">
         <v>163</v>
       </c>
@@ -15127,7 +15135,7 @@
         <v>TS-UD-DOC-CLS-001test_002_clause_creation_minimum_fields</v>
       </c>
     </row>
-    <row r="123" spans="1:11" ht="31.5" thickBot="1">
+    <row r="123" spans="1:11" ht="31.2" thickBot="1">
       <c r="A123" s="4" t="s">
         <v>163</v>
       </c>
@@ -15156,7 +15164,7 @@
         <v>TS-UD-DOC-CLS-001test_003_clause_creation_fails_without_content</v>
       </c>
     </row>
-    <row r="124" spans="1:11" ht="31.5" thickBot="1">
+    <row r="124" spans="1:11" ht="31.2" thickBot="1">
       <c r="A124" s="4" t="s">
         <v>163</v>
       </c>
@@ -15185,7 +15193,7 @@
         <v>TS-UD-DOC-CLS-001test_004_clause_creation_fails_without_document_id</v>
       </c>
     </row>
-    <row r="125" spans="1:11" ht="31.5" thickBot="1">
+    <row r="125" spans="1:11" ht="31.2" thickBot="1">
       <c r="A125" s="4" t="s">
         <v>163</v>
       </c>
@@ -15214,7 +15222,7 @@
         <v>TS-UD-DOC-CLS-001test_005_clause_creation_fails_without_tenant_id</v>
       </c>
     </row>
-    <row r="126" spans="1:11" ht="31.5" thickBot="1">
+    <row r="126" spans="1:11" ht="31.2" thickBot="1">
       <c r="A126" s="4" t="s">
         <v>163</v>
       </c>
@@ -15243,7 +15251,7 @@
         <v>TS-UD-DOC-CLS-001test_006_clause_immutability_after_creation</v>
       </c>
     </row>
-    <row r="127" spans="1:11" ht="31.5" thickBot="1">
+    <row r="127" spans="1:11" ht="31.2" thickBot="1">
       <c r="A127" s="4" t="s">
         <v>163</v>
       </c>
@@ -15272,7 +15280,7 @@
         <v>TS-UD-DOC-CLS-001test_007_clause_number_format_primera</v>
       </c>
     </row>
-    <row r="128" spans="1:11" ht="31.5" thickBot="1">
+    <row r="128" spans="1:11" ht="31.2" thickBot="1">
       <c r="A128" s="4" t="s">
         <v>163</v>
       </c>
@@ -15301,7 +15309,7 @@
         <v>TS-UD-DOC-CLS-001test_008_clause_number_format_numeric</v>
       </c>
     </row>
-    <row r="129" spans="1:11" ht="31.5" thickBot="1">
+    <row r="129" spans="1:11" ht="31.2" thickBot="1">
       <c r="A129" s="4" t="s">
         <v>163</v>
       </c>
@@ -15330,7 +15338,7 @@
         <v>TS-UD-DOC-CLS-001test_009_clause_number_format_decimal</v>
       </c>
     </row>
-    <row r="130" spans="1:11" ht="31.5" thickBot="1">
+    <row r="130" spans="1:11" ht="31.2" thickBot="1">
       <c r="A130" s="4" t="s">
         <v>163</v>
       </c>
@@ -15359,7 +15367,7 @@
         <v>TS-UD-DOC-CLS-001test_010_clause_number_normalization</v>
       </c>
     </row>
-    <row r="131" spans="1:11" ht="31.5" thickBot="1">
+    <row r="131" spans="1:11" ht="31.2" thickBot="1">
       <c r="A131" s="4" t="s">
         <v>163</v>
       </c>
@@ -15388,7 +15396,7 @@
         <v>TS-UD-DOC-CLS-001test_011_clause_content_max_length</v>
       </c>
     </row>
-    <row r="132" spans="1:11" ht="31.5" thickBot="1">
+    <row r="132" spans="1:11" ht="31.2" thickBot="1">
       <c r="A132" s="4" t="s">
         <v>163</v>
       </c>
@@ -15417,7 +15425,7 @@
         <v>TS-UD-DOC-CLS-001test_012_clause_content_empty_rejected</v>
       </c>
     </row>
-    <row r="133" spans="1:11" ht="31.5" thickBot="1">
+    <row r="133" spans="1:11" ht="31.2" thickBot="1">
       <c r="A133" s="4" t="s">
         <v>163</v>
       </c>
@@ -15446,7 +15454,7 @@
         <v>TS-UD-DOC-CLS-001test_013_clause_document_fk_valid</v>
       </c>
     </row>
-    <row r="134" spans="1:11" ht="31.5" thickBot="1">
+    <row r="134" spans="1:11" ht="31.2" thickBot="1">
       <c r="A134" s="4" t="s">
         <v>163</v>
       </c>
@@ -15475,7 +15483,7 @@
         <v>TS-UD-DOC-CLS-001test_014_clause_document_fk_invalid_rejected</v>
       </c>
     </row>
-    <row r="135" spans="1:11" ht="31.5" thickBot="1">
+    <row r="135" spans="1:11" ht="31.2" thickBot="1">
       <c r="A135" s="4" t="s">
         <v>163</v>
       </c>
@@ -15504,7 +15512,7 @@
         <v>TS-UD-DOC-CLS-001test_015_clause_tenant_fk_valid</v>
       </c>
     </row>
-    <row r="136" spans="1:11" ht="31.5" thickBot="1">
+    <row r="136" spans="1:11" ht="31.2" thickBot="1">
       <c r="A136" s="4" t="s">
         <v>163</v>
       </c>
@@ -15533,7 +15541,7 @@
         <v>TS-UD-DOC-CLS-001test_016_clause_tenant_fk_invalid_rejected</v>
       </c>
     </row>
-    <row r="137" spans="1:11" ht="31.5" thickBot="1">
+    <row r="137" spans="1:11" ht="31.2" thickBot="1">
       <c r="A137" s="4" t="s">
         <v>163</v>
       </c>
@@ -15562,7 +15570,7 @@
         <v>TS-UD-DOC-CLS-001test_017_clause_on_delete_restrict_document</v>
       </c>
     </row>
-    <row r="138" spans="1:11" ht="31.5" thickBot="1">
+    <row r="138" spans="1:11" ht="31.2" thickBot="1">
       <c r="A138" s="4" t="s">
         <v>163</v>
       </c>
@@ -15591,7 +15599,7 @@
         <v>TS-UD-DOC-CLS-001test_018_clause_on_delete_restrict_tenant</v>
       </c>
     </row>
-    <row r="139" spans="1:11" ht="31.5" thickBot="1">
+    <row r="139" spans="1:11" ht="31.2" thickBot="1">
       <c r="A139" s="4" t="s">
         <v>163</v>
       </c>
@@ -15620,7 +15628,7 @@
         <v>TS-UD-DOC-CLS-001test_019_clause_embedding_vector_size</v>
       </c>
     </row>
-    <row r="140" spans="1:11" ht="31.5" thickBot="1">
+    <row r="140" spans="1:11" ht="31.2" thickBot="1">
       <c r="A140" s="4" t="s">
         <v>163</v>
       </c>
@@ -15649,7 +15657,7 @@
         <v>TS-UD-DOC-CLS-001test_020_clause_embedding_generation</v>
       </c>
     </row>
-    <row r="141" spans="1:11" ht="31.5" thickBot="1">
+    <row r="141" spans="1:11" ht="31.2" thickBot="1">
       <c r="A141" s="4" t="s">
         <v>163</v>
       </c>
@@ -15678,7 +15686,7 @@
         <v>TS-UD-DOC-CLS-001test_021_clause_embedding_null_allowed</v>
       </c>
     </row>
-    <row r="142" spans="1:11" ht="31.5" thickBot="1">
+    <row r="142" spans="1:11" ht="31.2" thickBot="1">
       <c r="A142" s="4" t="s">
         <v>163</v>
       </c>
@@ -15707,7 +15715,7 @@
         <v>TS-UD-DOC-CLS-001test_022_clause_embedding_update</v>
       </c>
     </row>
-    <row r="143" spans="1:11" ht="16.5" thickBot="1">
+    <row r="143" spans="1:11" ht="16.2" thickBot="1">
       <c r="A143" s="4" t="s">
         <v>189</v>
       </c>
@@ -15736,7 +15744,7 @@
         <v>TS-UD-DOC-CLS-002Tests not individually listed</v>
       </c>
     </row>
-    <row r="144" spans="1:11" ht="16.5" thickBot="1">
+    <row r="144" spans="1:11" ht="16.2" thickBot="1">
       <c r="A144" s="4" t="s">
         <v>191</v>
       </c>
@@ -15762,7 +15770,7 @@
         <v>TS-UD-DOC-CLS-003Tests not individually listed</v>
       </c>
     </row>
-    <row r="145" spans="1:11" ht="31.5" thickBot="1">
+    <row r="145" spans="1:11" ht="31.2" thickBot="1">
       <c r="A145" s="4" t="s">
         <v>192</v>
       </c>
@@ -15791,7 +15799,7 @@
         <v>TS-UD-DOC-ENT-001test_001_date_dd_mm_yyyy_slash</v>
       </c>
     </row>
-    <row r="146" spans="1:11" ht="31.5" thickBot="1">
+    <row r="146" spans="1:11" ht="31.2" thickBot="1">
       <c r="A146" s="4" t="s">
         <v>192</v>
       </c>
@@ -15820,7 +15828,7 @@
         <v>TS-UD-DOC-ENT-001test_002_date_yyyy_mm_dd_dash</v>
       </c>
     </row>
-    <row r="147" spans="1:11" ht="31.5" thickBot="1">
+    <row r="147" spans="1:11" ht="31.2" thickBot="1">
       <c r="A147" s="4" t="s">
         <v>192</v>
       </c>
@@ -15849,7 +15857,7 @@
         <v>TS-UD-DOC-ENT-001test_003_date_dd_month_yyyy_spanish</v>
       </c>
     </row>
-    <row r="148" spans="1:11" ht="31.5" thickBot="1">
+    <row r="148" spans="1:11" ht="31.2" thickBot="1">
       <c r="A148" s="4" t="s">
         <v>192</v>
       </c>
@@ -15878,7 +15886,7 @@
         <v>TS-UD-DOC-ENT-001test_004_date_month_dd_yyyy_english</v>
       </c>
     </row>
-    <row r="149" spans="1:11" ht="31.5" thickBot="1">
+    <row r="149" spans="1:11" ht="31.2" thickBot="1">
       <c r="A149" s="4" t="s">
         <v>192</v>
       </c>
@@ -15907,7 +15915,7 @@
         <v>TS-UD-DOC-ENT-001test_005_date_relative_30_days</v>
       </c>
     </row>
-    <row r="150" spans="1:11" ht="31.5" thickBot="1">
+    <row r="150" spans="1:11" ht="31.2" thickBot="1">
       <c r="A150" s="4" t="s">
         <v>192</v>
       </c>
@@ -15936,7 +15944,7 @@
         <v>TS-UD-DOC-ENT-001test_006_date_relative_3_months</v>
       </c>
     </row>
-    <row r="151" spans="1:11" ht="31.5" thickBot="1">
+    <row r="151" spans="1:11" ht="31.2" thickBot="1">
       <c r="A151" s="4" t="s">
         <v>192</v>
       </c>
@@ -15965,7 +15973,7 @@
         <v>TS-UD-DOC-ENT-001test_007_date_relative_1_year</v>
       </c>
     </row>
-    <row r="152" spans="1:11" ht="31.5" thickBot="1">
+    <row r="152" spans="1:11" ht="31.2" thickBot="1">
       <c r="A152" s="4" t="s">
         <v>192</v>
       </c>
@@ -15994,7 +16002,7 @@
         <v>TS-UD-DOC-ENT-001test_008_date_relative_from_date</v>
       </c>
     </row>
-    <row r="153" spans="1:11" ht="31.5" thickBot="1">
+    <row r="153" spans="1:11" ht="31.2" thickBot="1">
       <c r="A153" s="4" t="s">
         <v>192</v>
       </c>
@@ -16023,7 +16031,7 @@
         <v>TS-UD-DOC-ENT-001test_009_date_context_entrega</v>
       </c>
     </row>
-    <row r="154" spans="1:11" ht="31.5" thickBot="1">
+    <row r="154" spans="1:11" ht="31.2" thickBot="1">
       <c r="A154" s="4" t="s">
         <v>192</v>
       </c>
@@ -16052,7 +16060,7 @@
         <v>TS-UD-DOC-ENT-001test_010_date_context_firma</v>
       </c>
     </row>
-    <row r="155" spans="1:11" ht="31.5" thickBot="1">
+    <row r="155" spans="1:11" ht="31.2" thickBot="1">
       <c r="A155" s="4" t="s">
         <v>192</v>
       </c>
@@ -16081,7 +16089,7 @@
         <v>TS-UD-DOC-ENT-001test_011_date_context_inicio</v>
       </c>
     </row>
-    <row r="156" spans="1:11" ht="16.5" thickBot="1">
+    <row r="156" spans="1:11" ht="16.2" thickBot="1">
       <c r="A156" s="4" t="s">
         <v>192</v>
       </c>
@@ -16110,7 +16118,7 @@
         <v>TS-UD-DOC-ENT-001test_012_date_context_fin</v>
       </c>
     </row>
-    <row r="157" spans="1:11" ht="31.5" thickBot="1">
+    <row r="157" spans="1:11" ht="31.2" thickBot="1">
       <c r="A157" s="4" t="s">
         <v>192</v>
       </c>
@@ -16139,7 +16147,7 @@
         <v>TS-UD-DOC-ENT-001test_013_multiple_dates_extraction</v>
       </c>
     </row>
-    <row r="158" spans="1:11" ht="31.5" thickBot="1">
+    <row r="158" spans="1:11" ht="31.2" thickBot="1">
       <c r="A158" s="4" t="s">
         <v>192</v>
       </c>
@@ -16168,7 +16176,7 @@
         <v>TS-UD-DOC-ENT-001test_014_multiple_dates_ordering</v>
       </c>
     </row>
-    <row r="159" spans="1:11" ht="31.5" thickBot="1">
+    <row r="159" spans="1:11" ht="31.2" thickBot="1">
       <c r="A159" s="4" t="s">
         <v>192</v>
       </c>
@@ -16197,7 +16205,7 @@
         <v>TS-UD-DOC-ENT-001test_015_date_range_extraction</v>
       </c>
     </row>
-    <row r="160" spans="1:11" ht="31.5" thickBot="1">
+    <row r="160" spans="1:11" ht="31.2" thickBot="1">
       <c r="A160" s="4" t="s">
         <v>192</v>
       </c>
@@ -16226,7 +16234,7 @@
         <v>TS-UD-DOC-ENT-001test_016_date_invalid_format_ignored</v>
       </c>
     </row>
-    <row r="161" spans="1:11" ht="31.5" thickBot="1">
+    <row r="161" spans="1:11" ht="31.2" thickBot="1">
       <c r="A161" s="4" t="s">
         <v>210</v>
       </c>
@@ -16255,7 +16263,7 @@
         <v>TS-UD-DOC-ENT-002test_001_money_eur_symbol_suffix</v>
       </c>
     </row>
-    <row r="162" spans="1:11" ht="31.5" thickBot="1">
+    <row r="162" spans="1:11" ht="31.2" thickBot="1">
       <c r="A162" s="4" t="s">
         <v>210</v>
       </c>
@@ -16284,7 +16292,7 @@
         <v>TS-UD-DOC-ENT-002test_002_money_eur_symbol_prefix</v>
       </c>
     </row>
-    <row r="163" spans="1:11" ht="31.5" thickBot="1">
+    <row r="163" spans="1:11" ht="31.2" thickBot="1">
       <c r="A163" s="4" t="s">
         <v>210</v>
       </c>
@@ -16313,7 +16321,7 @@
         <v>TS-UD-DOC-ENT-002test_003_money_eur_word_euros</v>
       </c>
     </row>
-    <row r="164" spans="1:11" ht="31.5" thickBot="1">
+    <row r="164" spans="1:11" ht="31.2" thickBot="1">
       <c r="A164" s="4" t="s">
         <v>210</v>
       </c>
@@ -16342,7 +16350,7 @@
         <v>TS-UD-DOC-ENT-002test_004_money_eur_thousands_separator</v>
       </c>
     </row>
-    <row r="165" spans="1:11" ht="31.5" thickBot="1">
+    <row r="165" spans="1:11" ht="31.2" thickBot="1">
       <c r="A165" s="4" t="s">
         <v>210</v>
       </c>
@@ -16371,7 +16379,7 @@
         <v>TS-UD-DOC-ENT-002test_005_money_usd_symbol</v>
       </c>
     </row>
-    <row r="166" spans="1:11" ht="31.5" thickBot="1">
+    <row r="166" spans="1:11" ht="16.2" thickBot="1">
       <c r="A166" s="4" t="s">
         <v>210</v>
       </c>
@@ -16400,7 +16408,7 @@
         <v>TS-UD-DOC-ENT-002test_006_money_usd_word</v>
       </c>
     </row>
-    <row r="167" spans="1:11" ht="31.5" thickBot="1">
+    <row r="167" spans="1:11" ht="31.2" thickBot="1">
       <c r="A167" s="4" t="s">
         <v>210</v>
       </c>
@@ -16429,7 +16437,7 @@
         <v>TS-UD-DOC-ENT-002test_007_money_usd_thousands_separator</v>
       </c>
     </row>
-    <row r="168" spans="1:11" ht="31.5" thickBot="1">
+    <row r="168" spans="1:11" ht="31.2" thickBot="1">
       <c r="A168" s="4" t="s">
         <v>210</v>
       </c>
@@ -16458,7 +16466,7 @@
         <v>TS-UD-DOC-ENT-002test_008_money_context_anticipo</v>
       </c>
     </row>
-    <row r="169" spans="1:11" ht="31.5" thickBot="1">
+    <row r="169" spans="1:11" ht="31.2" thickBot="1">
       <c r="A169" s="4" t="s">
         <v>210</v>
       </c>
@@ -16487,7 +16495,7 @@
         <v>TS-UD-DOC-ENT-002test_009_money_context_pago_final</v>
       </c>
     </row>
-    <row r="170" spans="1:11" ht="31.5" thickBot="1">
+    <row r="170" spans="1:11" ht="31.2" thickBot="1">
       <c r="A170" s="4" t="s">
         <v>210</v>
       </c>
@@ -16516,7 +16524,7 @@
         <v>TS-UD-DOC-ENT-002test_010_money_context_penalizacion</v>
       </c>
     </row>
-    <row r="171" spans="1:11" ht="31.5" thickBot="1">
+    <row r="171" spans="1:11" ht="31.2" thickBot="1">
       <c r="A171" s="4" t="s">
         <v>210</v>
       </c>
@@ -16545,7 +16553,7 @@
         <v>TS-UD-DOC-ENT-002test_011_money_context_total</v>
       </c>
     </row>
-    <row r="172" spans="1:11" ht="31.5" thickBot="1">
+    <row r="172" spans="1:11" ht="31.2" thickBot="1">
       <c r="A172" s="4" t="s">
         <v>210</v>
       </c>
@@ -16574,7 +16582,7 @@
         <v>TS-UD-DOC-ENT-002test_012_multiple_amounts_extraction</v>
       </c>
     </row>
-    <row r="173" spans="1:11" ht="31.5" thickBot="1">
+    <row r="173" spans="1:11" ht="31.2" thickBot="1">
       <c r="A173" s="4" t="s">
         <v>210</v>
       </c>
@@ -16603,7 +16611,7 @@
         <v>TS-UD-DOC-ENT-002test_013_money_percentage_extraction</v>
       </c>
     </row>
-    <row r="174" spans="1:11" ht="31.5" thickBot="1">
+    <row r="174" spans="1:11" ht="31.2" thickBot="1">
       <c r="A174" s="4" t="s">
         <v>210</v>
       </c>
@@ -16632,7 +16640,7 @@
         <v>TS-UD-DOC-ENT-002test_014_money_negative_amount</v>
       </c>
     </row>
-    <row r="175" spans="1:11" ht="16.5" thickBot="1">
+    <row r="175" spans="1:11" ht="16.2" thickBot="1">
       <c r="A175" s="4" t="s">
         <v>225</v>
       </c>
@@ -16653,7 +16661,7 @@
         <v>TS-UD-DOC-ENT-003Tests not individually listed</v>
       </c>
     </row>
-    <row r="176" spans="1:11" ht="16.5" thickBot="1">
+    <row r="176" spans="1:11" ht="16.2" thickBot="1">
       <c r="A176" s="4" t="s">
         <v>226</v>
       </c>
@@ -16674,7 +16682,7 @@
         <v>TS-UD-DOC-ENT-004Tests not individually listed</v>
       </c>
     </row>
-    <row r="177" spans="1:11" ht="16.5" thickBot="1">
+    <row r="177" spans="1:11" ht="16.2" thickBot="1">
       <c r="A177" s="4" t="s">
         <v>227</v>
       </c>
@@ -16695,7 +16703,7 @@
         <v>TS-UD-DOC-DOC-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="178" spans="1:11" ht="16.5" thickBot="1">
+    <row r="178" spans="1:11" ht="16.2" thickBot="1">
       <c r="A178" s="4" t="s">
         <v>228</v>
       </c>
@@ -16716,7 +16724,7 @@
         <v>TS-UD-DOC-CNF-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="179" spans="1:11" ht="31.5" thickBot="1">
+    <row r="179" spans="1:11" ht="31.2" thickBot="1">
       <c r="A179" s="4" t="s">
         <v>229</v>
       </c>
@@ -16737,7 +16745,7 @@
         <v>TS-UD-COH-CAT-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="180" spans="1:11" ht="31.5" thickBot="1">
+    <row r="180" spans="1:11" ht="31.2" thickBot="1">
       <c r="A180" s="4" t="s">
         <v>231</v>
       </c>
@@ -16769,7 +16777,7 @@
         <v>TS-UD-COH-RUL-001test_001_r11_wbs_level4_no_activities_alert</v>
       </c>
     </row>
-    <row r="181" spans="1:11" ht="31.5" thickBot="1">
+    <row r="181" spans="1:11" ht="31.2" thickBot="1">
       <c r="A181" s="4" t="s">
         <v>231</v>
       </c>
@@ -16798,7 +16806,7 @@
         <v>TS-UD-COH-RUL-001test_002_r11_wbs_level4_with_activities_pass</v>
       </c>
     </row>
-    <row r="182" spans="1:11" ht="31.5" thickBot="1">
+    <row r="182" spans="1:11" ht="31.2" thickBot="1">
       <c r="A182" s="4" t="s">
         <v>231</v>
       </c>
@@ -16827,7 +16835,7 @@
         <v>TS-UD-COH-RUL-001test_003_r11_wbs_level3_no_activities_ignored</v>
       </c>
     </row>
-    <row r="183" spans="1:11" ht="31.5" thickBot="1">
+    <row r="183" spans="1:11" ht="31.2" thickBot="1">
       <c r="A183" s="4" t="s">
         <v>231</v>
       </c>
@@ -16856,7 +16864,7 @@
         <v>TS-UD-COH-RUL-001test_004_r11_wbs_level2_no_activities_ignored</v>
       </c>
     </row>
-    <row r="184" spans="1:11" ht="31.5" thickBot="1">
+    <row r="184" spans="1:11" ht="31.2" thickBot="1">
       <c r="A184" s="4" t="s">
         <v>231</v>
       </c>
@@ -16885,7 +16893,7 @@
         <v>TS-UD-COH-RUL-001test_005_r11_multiple_wbs_level4_violations</v>
       </c>
     </row>
-    <row r="185" spans="1:11" ht="31.5" thickBot="1">
+    <row r="185" spans="1:11" ht="31.2" thickBot="1">
       <c r="A185" s="4" t="s">
         <v>231</v>
       </c>
@@ -16914,7 +16922,7 @@
         <v>TS-UD-COH-RUL-001test_006_r11_alert_severity_medium</v>
       </c>
     </row>
-    <row r="186" spans="1:11" ht="31.5" thickBot="1">
+    <row r="186" spans="1:11" ht="31.2" thickBot="1">
       <c r="A186" s="4" t="s">
         <v>231</v>
       </c>
@@ -16943,7 +16951,7 @@
         <v>TS-UD-COH-RUL-001test_007_r12_wbs_no_budget_line_alert</v>
       </c>
     </row>
-    <row r="187" spans="1:11" ht="31.5" thickBot="1">
+    <row r="187" spans="1:11" ht="31.2" thickBot="1">
       <c r="A187" s="4" t="s">
         <v>231</v>
       </c>
@@ -16972,7 +16980,7 @@
         <v>TS-UD-COH-RUL-001test_008_r12_wbs_with_budget_line_pass</v>
       </c>
     </row>
-    <row r="188" spans="1:11" ht="31.5" thickBot="1">
+    <row r="188" spans="1:11" ht="31.2" thickBot="1">
       <c r="A188" s="4" t="s">
         <v>231</v>
       </c>
@@ -17001,7 +17009,7 @@
         <v>TS-UD-COH-RUL-001test_009_r12_wbs_budget_zero_warning</v>
       </c>
     </row>
-    <row r="189" spans="1:11" ht="31.5" thickBot="1">
+    <row r="189" spans="1:11" ht="31.2" thickBot="1">
       <c r="A189" s="4" t="s">
         <v>231</v>
       </c>
@@ -17030,7 +17038,7 @@
         <v>TS-UD-COH-RUL-001test_010_r12_multiple_wbs_violations</v>
       </c>
     </row>
-    <row r="190" spans="1:11" ht="31.5" thickBot="1">
+    <row r="190" spans="1:11" ht="31.2" thickBot="1">
       <c r="A190" s="4" t="s">
         <v>231</v>
       </c>
@@ -17059,7 +17067,7 @@
         <v>TS-UD-COH-RUL-001test_011_r12_alert_severity_high</v>
       </c>
     </row>
-    <row r="191" spans="1:11" ht="31.5" thickBot="1">
+    <row r="191" spans="1:11" ht="31.2" thickBot="1">
       <c r="A191" s="4" t="s">
         <v>231</v>
       </c>
@@ -17088,7 +17096,7 @@
         <v>TS-UD-COH-RUL-001test_012_r12_affected_entities_list</v>
       </c>
     </row>
-    <row r="192" spans="1:11" ht="31.5" thickBot="1">
+    <row r="192" spans="1:11" ht="31.2" thickBot="1">
       <c r="A192" s="4" t="s">
         <v>231</v>
       </c>
@@ -17117,7 +17125,7 @@
         <v>TS-UD-COH-RUL-001test_013_r13_scope_clause_no_wbs_alert</v>
       </c>
     </row>
-    <row r="193" spans="1:11" ht="31.5" thickBot="1">
+    <row r="193" spans="1:11" ht="31.2" thickBot="1">
       <c r="A193" s="4" t="s">
         <v>231</v>
       </c>
@@ -17146,7 +17154,7 @@
         <v>TS-UD-COH-RUL-001test_014_r13_scope_clause_with_wbs_pass</v>
       </c>
     </row>
-    <row r="194" spans="1:11" ht="31.5" thickBot="1">
+    <row r="194" spans="1:11" ht="31.2" thickBot="1">
       <c r="A194" s="4" t="s">
         <v>231</v>
       </c>
@@ -17175,7 +17183,7 @@
         <v>TS-UD-COH-RUL-001test_015_r13_partial_coverage_calculation</v>
       </c>
     </row>
-    <row r="195" spans="1:11" ht="31.5" thickBot="1">
+    <row r="195" spans="1:11" ht="31.2" thickBot="1">
       <c r="A195" s="4" t="s">
         <v>231</v>
       </c>
@@ -17204,7 +17212,7 @@
         <v>TS-UD-COH-RUL-001test_016_r13_coverage_percentage_80</v>
       </c>
     </row>
-    <row r="196" spans="1:11" ht="31.5" thickBot="1">
+    <row r="196" spans="1:11" ht="31.2" thickBot="1">
       <c r="A196" s="4" t="s">
         <v>231</v>
       </c>
@@ -17233,7 +17241,7 @@
         <v>TS-UD-COH-RUL-001test_017_r13_uncovered_clauses_list</v>
       </c>
     </row>
-    <row r="197" spans="1:11" ht="31.5" thickBot="1">
+    <row r="197" spans="1:11" ht="31.2" thickBot="1">
       <c r="A197" s="4" t="s">
         <v>231</v>
       </c>
@@ -17262,7 +17270,7 @@
         <v>TS-UD-COH-RUL-001test_018_r13_alert_severity_high</v>
       </c>
     </row>
-    <row r="198" spans="1:11" ht="31.5" thickBot="1">
+    <row r="198" spans="1:11" ht="31.2" thickBot="1">
       <c r="A198" s="4" t="s">
         <v>253</v>
       </c>
@@ -17291,7 +17299,7 @@
         <v>TS-UD-COH-RUL-002test_001_r6_deviation_10_percent_alert</v>
       </c>
     </row>
-    <row r="199" spans="1:11" ht="31.5" thickBot="1">
+    <row r="199" spans="1:11" ht="31.2" thickBot="1">
       <c r="A199" s="4" t="s">
         <v>253</v>
       </c>
@@ -17320,7 +17328,7 @@
         <v>TS-UD-COH-RUL-002test_002_r6_deviation_5_percent_pass</v>
       </c>
     </row>
-    <row r="200" spans="1:11" ht="31.5" thickBot="1">
+    <row r="200" spans="1:11" ht="31.2" thickBot="1">
       <c r="A200" s="4" t="s">
         <v>253</v>
       </c>
@@ -17349,7 +17357,7 @@
         <v>TS-UD-COH-RUL-002test_003_r6_deviation_4_9_percent_pass</v>
       </c>
     </row>
-    <row r="201" spans="1:11" ht="31.5" thickBot="1">
+    <row r="201" spans="1:11" ht="31.2" thickBot="1">
       <c r="A201" s="4" t="s">
         <v>253</v>
       </c>
@@ -17378,7 +17386,7 @@
         <v>TS-UD-COH-RUL-002test_004_r6_over_budget_critical</v>
       </c>
     </row>
-    <row r="202" spans="1:11" ht="31.5" thickBot="1">
+    <row r="202" spans="1:11" ht="31.2" thickBot="1">
       <c r="A202" s="4" t="s">
         <v>253</v>
       </c>
@@ -17407,7 +17415,7 @@
         <v>TS-UD-COH-RUL-002test_005_r6_under_budget_warning</v>
       </c>
     </row>
-    <row r="203" spans="1:11" ht="31.5" thickBot="1">
+    <row r="203" spans="1:11" ht="31.2" thickBot="1">
       <c r="A203" s="4" t="s">
         <v>253</v>
       </c>
@@ -17436,7 +17444,7 @@
         <v>TS-UD-COH-RUL-002test_006_r6_exact_match_pass</v>
       </c>
     </row>
-    <row r="204" spans="1:11" ht="31.5" thickBot="1">
+    <row r="204" spans="1:11" ht="31.2" thickBot="1">
       <c r="A204" s="4" t="s">
         <v>253</v>
       </c>
@@ -17465,7 +17473,7 @@
         <v>TS-UD-COH-RUL-002test_007_r15_bom_no_budget_alert</v>
       </c>
     </row>
-    <row r="205" spans="1:11" ht="31.5" thickBot="1">
+    <row r="205" spans="1:11" ht="31.2" thickBot="1">
       <c r="A205" s="4" t="s">
         <v>253</v>
       </c>
@@ -17494,7 +17502,7 @@
         <v>TS-UD-COH-RUL-002test_008_r15_bom_with_budget_pass</v>
       </c>
     </row>
-    <row r="206" spans="1:11" ht="31.5" thickBot="1">
+    <row r="206" spans="1:11" ht="31.2" thickBot="1">
       <c r="A206" s="4" t="s">
         <v>253</v>
       </c>
@@ -17523,7 +17531,7 @@
         <v>TS-UD-COH-RUL-002test_009_r15_bom_client_provided_exception</v>
       </c>
     </row>
-    <row r="207" spans="1:11" ht="31.5" thickBot="1">
+    <row r="207" spans="1:11" ht="31.2" thickBot="1">
       <c r="A207" s="4" t="s">
         <v>253</v>
       </c>
@@ -17552,7 +17560,7 @@
         <v>TS-UD-COH-RUL-002test_010_r15_multiple_bom_violations</v>
       </c>
     </row>
-    <row r="208" spans="1:11" ht="31.5" thickBot="1">
+    <row r="208" spans="1:11" ht="31.2" thickBot="1">
       <c r="A208" s="4" t="s">
         <v>253</v>
       </c>
@@ -17581,7 +17589,7 @@
         <v>TS-UD-COH-RUL-002test_011_r15_affected_items_list</v>
       </c>
     </row>
-    <row r="209" spans="1:11" ht="31.5" thickBot="1">
+    <row r="209" spans="1:11" ht="31.2" thickBot="1">
       <c r="A209" s="4" t="s">
         <v>253</v>
       </c>
@@ -17610,7 +17618,7 @@
         <v>TS-UD-COH-RUL-002test_012_r16_deviation_11_percent_alert</v>
       </c>
     </row>
-    <row r="210" spans="1:11" ht="31.5" thickBot="1">
+    <row r="210" spans="1:11" ht="31.2" thickBot="1">
       <c r="A210" s="4" t="s">
         <v>253</v>
       </c>
@@ -17639,7 +17647,7 @@
         <v>TS-UD-COH-RUL-002test_013_r16_deviation_10_percent_pass</v>
       </c>
     </row>
-    <row r="211" spans="1:11" ht="31.5" thickBot="1">
+    <row r="211" spans="1:11" ht="31.2" thickBot="1">
       <c r="A211" s="4" t="s">
         <v>253</v>
       </c>
@@ -17668,7 +17676,7 @@
         <v>TS-UD-COH-RUL-002test_014_r16_over_budget_critical</v>
       </c>
     </row>
-    <row r="212" spans="1:11" ht="31.5" thickBot="1">
+    <row r="212" spans="1:11" ht="31.2" thickBot="1">
       <c r="A212" s="4" t="s">
         <v>253</v>
       </c>
@@ -17697,7 +17705,7 @@
         <v>TS-UD-COH-RUL-002test_015_r16_under_budget_different_severity</v>
       </c>
     </row>
-    <row r="213" spans="1:11" ht="31.5" thickBot="1">
+    <row r="213" spans="1:11" ht="31.2" thickBot="1">
       <c r="A213" s="4" t="s">
         <v>253</v>
       </c>
@@ -17726,7 +17734,7 @@
         <v>TS-UD-COH-RUL-002test_016_r16_trend_calculation</v>
       </c>
     </row>
-    <row r="214" spans="1:11" ht="31.5" thickBot="1">
+    <row r="214" spans="1:11" ht="31.2" thickBot="1">
       <c r="A214" s="4" t="s">
         <v>270</v>
       </c>
@@ -17758,7 +17766,7 @@
         <v>TS-UD-COH-RUL-003test_001_r1_dates_mismatch_alert</v>
       </c>
     </row>
-    <row r="215" spans="1:11" ht="31.5" thickBot="1">
+    <row r="215" spans="1:11" ht="31.2" thickBot="1">
       <c r="A215" s="4" t="s">
         <v>270</v>
       </c>
@@ -17787,7 +17795,7 @@
         <v>TS-UD-COH-RUL-003test_002_r1_dates_match_pass</v>
       </c>
     </row>
-    <row r="216" spans="1:11" ht="31.5" thickBot="1">
+    <row r="216" spans="1:11" ht="31.2" thickBot="1">
       <c r="A216" s="4" t="s">
         <v>270</v>
       </c>
@@ -17816,7 +17824,7 @@
         <v>TS-UD-COH-RUL-003test_003_r1_schedule_late_critical</v>
       </c>
     </row>
-    <row r="217" spans="1:11" ht="31.5" thickBot="1">
+    <row r="217" spans="1:11" ht="31.2" thickBot="1">
       <c r="A217" s="4" t="s">
         <v>270</v>
       </c>
@@ -17845,7 +17853,7 @@
         <v>TS-UD-COH-RUL-003test_004_r1_schedule_early_warning</v>
       </c>
     </row>
-    <row r="218" spans="1:11" ht="31.5" thickBot="1">
+    <row r="218" spans="1:11" ht="31.2" thickBot="1">
       <c r="A218" s="4" t="s">
         <v>270</v>
       </c>
@@ -17874,7 +17882,7 @@
         <v>TS-UD-COH-RUL-003test_005_r1_delta_days_calculation</v>
       </c>
     </row>
-    <row r="219" spans="1:11" ht="31.5" thickBot="1">
+    <row r="219" spans="1:11" ht="31.2" thickBot="1">
       <c r="A219" s="4" t="s">
         <v>270</v>
       </c>
@@ -17903,7 +17911,7 @@
         <v>TS-UD-COH-RUL-003test_006_r2_milestone_no_activity_alert</v>
       </c>
     </row>
-    <row r="220" spans="1:11" ht="31.5" thickBot="1">
+    <row r="220" spans="1:11" ht="31.2" thickBot="1">
       <c r="A220" s="4" t="s">
         <v>270</v>
       </c>
@@ -17932,7 +17940,7 @@
         <v>TS-UD-COH-RUL-003test_007_r2_milestone_with_activity_pass</v>
       </c>
     </row>
-    <row r="221" spans="1:11" ht="31.5" thickBot="1">
+    <row r="221" spans="1:11" ht="31.2" thickBot="1">
       <c r="A221" s="4" t="s">
         <v>270</v>
       </c>
@@ -17961,7 +17969,7 @@
         <v>TS-UD-COH-RUL-003test_008_r2_milestone_date_mismatch_alert</v>
       </c>
     </row>
-    <row r="222" spans="1:11" ht="31.5" thickBot="1">
+    <row r="222" spans="1:11" ht="31.2" thickBot="1">
       <c r="A222" s="4" t="s">
         <v>270</v>
       </c>
@@ -17990,7 +17998,7 @@
         <v>TS-UD-COH-RUL-003test_009_r2_multiple_milestones_violations</v>
       </c>
     </row>
-    <row r="223" spans="1:11" ht="31.5" thickBot="1">
+    <row r="223" spans="1:11" ht="31.2" thickBot="1">
       <c r="A223" s="4" t="s">
         <v>270</v>
       </c>
@@ -18019,7 +18027,7 @@
         <v>TS-UD-COH-RUL-003test_010_r2_unlinked_milestones_list</v>
       </c>
     </row>
-    <row r="224" spans="1:11" ht="31.5" thickBot="1">
+    <row r="224" spans="1:11" ht="31.2" thickBot="1">
       <c r="A224" s="4" t="s">
         <v>270</v>
       </c>
@@ -18048,7 +18056,7 @@
         <v>TS-UD-COH-RUL-003test_011_r5_activity_exceeds_contract_alert</v>
       </c>
     </row>
-    <row r="225" spans="1:11" ht="31.5" thickBot="1">
+    <row r="225" spans="1:11" ht="31.2" thickBot="1">
       <c r="A225" s="4" t="s">
         <v>270</v>
       </c>
@@ -18077,7 +18085,7 @@
         <v>TS-UD-COH-RUL-003test_012_r5_activity_within_contract_pass</v>
       </c>
     </row>
-    <row r="226" spans="1:11" ht="31.5" thickBot="1">
+    <row r="226" spans="1:11" ht="31.2" thickBot="1">
       <c r="A226" s="4" t="s">
         <v>270</v>
       </c>
@@ -18106,7 +18114,7 @@
         <v>TS-UD-COH-RUL-003test_013_r5_exceeding_activities_list</v>
       </c>
     </row>
-    <row r="227" spans="1:11" ht="31.5" thickBot="1">
+    <row r="227" spans="1:11" ht="31.2" thickBot="1">
       <c r="A227" s="4" t="s">
         <v>270</v>
       </c>
@@ -18135,7 +18143,7 @@
         <v>TS-UD-COH-RUL-003test_014_r5_alert_severity_critical</v>
       </c>
     </row>
-    <row r="228" spans="1:11" ht="31.5" thickBot="1">
+    <row r="228" spans="1:11" ht="31.2" thickBot="1">
       <c r="A228" s="4" t="s">
         <v>270</v>
       </c>
@@ -18164,7 +18172,7 @@
         <v>TS-UD-COH-RUL-003test_015_r14_order_date_passed_critical</v>
       </c>
     </row>
-    <row r="229" spans="1:11" ht="31.5" thickBot="1">
+    <row r="229" spans="1:11" ht="31.2" thickBot="1">
       <c r="A229" s="4" t="s">
         <v>270</v>
       </c>
@@ -18193,7 +18201,7 @@
         <v>TS-UD-COH-RUL-003test_016_r14_order_date_tight_warning</v>
       </c>
     </row>
-    <row r="230" spans="1:11" ht="31.5" thickBot="1">
+    <row r="230" spans="1:11" ht="31.2" thickBot="1">
       <c r="A230" s="4" t="s">
         <v>288</v>
       </c>
@@ -18214,7 +18222,7 @@
         <v>TS-UD-COH-RUL-004Tests not individually listed</v>
       </c>
     </row>
-    <row r="231" spans="1:11" ht="31.5" thickBot="1">
+    <row r="231" spans="1:11" ht="31.2" thickBot="1">
       <c r="A231" s="4" t="s">
         <v>289</v>
       </c>
@@ -18235,7 +18243,7 @@
         <v>TS-UD-COH-RUL-005Tests not individually listed</v>
       </c>
     </row>
-    <row r="232" spans="1:11" ht="31.5" thickBot="1">
+    <row r="232" spans="1:11" ht="31.2" thickBot="1">
       <c r="A232" s="4" t="s">
         <v>290</v>
       </c>
@@ -18256,7 +18264,7 @@
         <v>TS-UD-COH-RUL-006Tests not individually listed</v>
       </c>
     </row>
-    <row r="233" spans="1:11" ht="31.5" thickBot="1">
+    <row r="233" spans="1:11" ht="31.2" thickBot="1">
       <c r="A233" s="4" t="s">
         <v>291</v>
       </c>
@@ -18288,7 +18296,7 @@
         <v>TS-UD-COH-SCR-001test_001_subscore_no_alerts_100_percent</v>
       </c>
     </row>
-    <row r="234" spans="1:11" ht="31.5" thickBot="1">
+    <row r="234" spans="1:11" ht="31.2" thickBot="1">
       <c r="A234" s="4" t="s">
         <v>291</v>
       </c>
@@ -18317,7 +18325,7 @@
         <v>TS-UD-COH-SCR-001test_002_subscore_one_alert_penalized</v>
       </c>
     </row>
-    <row r="235" spans="1:11" ht="31.5" thickBot="1">
+    <row r="235" spans="1:11" ht="31.2" thickBot="1">
       <c r="A235" s="4" t="s">
         <v>291</v>
       </c>
@@ -18346,7 +18354,7 @@
         <v>TS-UD-COH-SCR-001test_003_subscore_multiple_alerts_cumulative</v>
       </c>
     </row>
-    <row r="236" spans="1:11" ht="31.5" thickBot="1">
+    <row r="236" spans="1:11" ht="31.2" thickBot="1">
       <c r="A236" s="4" t="s">
         <v>291</v>
       </c>
@@ -18375,7 +18383,7 @@
         <v>TS-UD-COH-SCR-001test_004_subscore_severity_low_penalty_5</v>
       </c>
     </row>
-    <row r="237" spans="1:11" ht="31.5" thickBot="1">
+    <row r="237" spans="1:11" ht="31.2" thickBot="1">
       <c r="A237" s="4" t="s">
         <v>291</v>
       </c>
@@ -18404,7 +18412,7 @@
         <v>TS-UD-COH-SCR-001test_005_subscore_severity_medium_penalty_10</v>
       </c>
     </row>
-    <row r="238" spans="1:11" ht="31.5" thickBot="1">
+    <row r="238" spans="1:11" ht="31.2" thickBot="1">
       <c r="A238" s="4" t="s">
         <v>291</v>
       </c>
@@ -18433,7 +18441,7 @@
         <v>TS-UD-COH-SCR-001test_006_subscore_severity_high_penalty_20</v>
       </c>
     </row>
-    <row r="239" spans="1:11" ht="31.5" thickBot="1">
+    <row r="239" spans="1:11" ht="31.2" thickBot="1">
       <c r="A239" s="4" t="s">
         <v>291</v>
       </c>
@@ -18462,7 +18470,7 @@
         <v>TS-UD-COH-SCR-001test_007_subscore_severity_critical_penalty_30</v>
       </c>
     </row>
-    <row r="240" spans="1:11" ht="31.5" thickBot="1">
+    <row r="240" spans="1:11" ht="31.2" thickBot="1">
       <c r="A240" s="4" t="s">
         <v>291</v>
       </c>
@@ -18491,7 +18499,7 @@
         <v>TS-UD-COH-SCR-001test_008_subscore_scope_calculation</v>
       </c>
     </row>
-    <row r="241" spans="1:11" ht="31.5" thickBot="1">
+    <row r="241" spans="1:11" ht="31.2" thickBot="1">
       <c r="A241" s="4" t="s">
         <v>291</v>
       </c>
@@ -18520,7 +18528,7 @@
         <v>TS-UD-COH-SCR-001test_009_subscore_budget_calculation</v>
       </c>
     </row>
-    <row r="242" spans="1:11" ht="31.5" thickBot="1">
+    <row r="242" spans="1:11" ht="31.2" thickBot="1">
       <c r="A242" s="4" t="s">
         <v>291</v>
       </c>
@@ -18549,7 +18557,7 @@
         <v>TS-UD-COH-SCR-001test_010_subscore_quality_calculation</v>
       </c>
     </row>
-    <row r="243" spans="1:11" ht="31.5" thickBot="1">
+    <row r="243" spans="1:11" ht="31.2" thickBot="1">
       <c r="A243" s="4" t="s">
         <v>291</v>
       </c>
@@ -18578,7 +18586,7 @@
         <v>TS-UD-COH-SCR-001test_011_subscore_technical_calculation</v>
       </c>
     </row>
-    <row r="244" spans="1:11" ht="31.5" thickBot="1">
+    <row r="244" spans="1:11" ht="31.2" thickBot="1">
       <c r="A244" s="4" t="s">
         <v>291</v>
       </c>
@@ -18607,7 +18615,7 @@
         <v>TS-UD-COH-SCR-001test_012_subscore_legal_calculation</v>
       </c>
     </row>
-    <row r="245" spans="1:11" ht="31.5" thickBot="1">
+    <row r="245" spans="1:11" ht="31.2" thickBot="1">
       <c r="A245" s="4" t="s">
         <v>291</v>
       </c>
@@ -18636,7 +18644,7 @@
         <v>TS-UD-COH-SCR-001test_013_subscore_time_calculation</v>
       </c>
     </row>
-    <row r="246" spans="1:11" ht="31.5" thickBot="1">
+    <row r="246" spans="1:11" ht="31.2" thickBot="1">
       <c r="A246" s="4" t="s">
         <v>291</v>
       </c>
@@ -18665,7 +18673,7 @@
         <v>TS-UD-COH-SCR-001test_014_subscore_floor_at_zero</v>
       </c>
     </row>
-    <row r="247" spans="1:11" ht="31.5" thickBot="1">
+    <row r="247" spans="1:11" ht="31.2" thickBot="1">
       <c r="A247" s="4" t="s">
         <v>307</v>
       </c>
@@ -18694,7 +18702,7 @@
         <v>TS-UD-COH-SCR-002test_001_global_score_formula_verification</v>
       </c>
     </row>
-    <row r="248" spans="1:11" ht="31.5" thickBot="1">
+    <row r="248" spans="1:11" ht="31.2" thickBot="1">
       <c r="A248" s="4" t="s">
         <v>307</v>
       </c>
@@ -18723,7 +18731,7 @@
         <v>TS-UD-COH-SCR-002test_002_global_score_default_weights</v>
       </c>
     </row>
-    <row r="249" spans="1:11" ht="31.5" thickBot="1">
+    <row r="249" spans="1:11" ht="31.2" thickBot="1">
       <c r="A249" s="4" t="s">
         <v>307</v>
       </c>
@@ -18752,7 +18760,7 @@
         <v>TS-UD-COH-SCR-002test_003_global_score_all_100_equals_100</v>
       </c>
     </row>
-    <row r="250" spans="1:11" ht="31.5" thickBot="1">
+    <row r="250" spans="1:11" ht="31.2" thickBot="1">
       <c r="A250" s="4" t="s">
         <v>307</v>
       </c>
@@ -18781,7 +18789,7 @@
         <v>TS-UD-COH-SCR-002test_004_global_score_all_0_equals_0</v>
       </c>
     </row>
-    <row r="251" spans="1:11" ht="31.5" thickBot="1">
+    <row r="251" spans="1:11" ht="31.2" thickBot="1">
       <c r="A251" s="4" t="s">
         <v>307</v>
       </c>
@@ -18810,7 +18818,7 @@
         <v>TS-UD-COH-SCR-002test_005_global_score_mixed_subscores</v>
       </c>
     </row>
-    <row r="252" spans="1:11" ht="31.5" thickBot="1">
+    <row r="252" spans="1:11" ht="31.2" thickBot="1">
       <c r="A252" s="4" t="s">
         <v>307</v>
       </c>
@@ -18839,7 +18847,7 @@
         <v>TS-UD-COH-SCR-002test_006_global_score_range_0_to_100</v>
       </c>
     </row>
-    <row r="253" spans="1:11" ht="31.5" thickBot="1">
+    <row r="253" spans="1:11" ht="31.2" thickBot="1">
       <c r="A253" s="4" t="s">
         <v>307</v>
       </c>
@@ -18868,7 +18876,7 @@
         <v>TS-UD-COH-SCR-002test_007_weights_sum_validation</v>
       </c>
     </row>
-    <row r="254" spans="1:11" ht="31.5" thickBot="1">
+    <row r="254" spans="1:11" ht="31.2" thickBot="1">
       <c r="A254" s="4" t="s">
         <v>307</v>
       </c>
@@ -18897,7 +18905,7 @@
         <v>TS-UD-COH-SCR-002test_008_weights_normalization_auto</v>
       </c>
     </row>
-    <row r="255" spans="1:11" ht="31.5" thickBot="1">
+    <row r="255" spans="1:11" ht="31.2" thickBot="1">
       <c r="A255" s="4" t="s">
         <v>307</v>
       </c>
@@ -18926,7 +18934,7 @@
         <v>TS-UD-COH-SCR-002test_009_weights_custom_budget_30</v>
       </c>
     </row>
-    <row r="256" spans="1:11" ht="31.5" thickBot="1">
+    <row r="256" spans="1:11" ht="31.2" thickBot="1">
       <c r="A256" s="4" t="s">
         <v>307</v>
       </c>
@@ -18955,7 +18963,7 @@
         <v>TS-UD-COH-SCR-002test_010_weights_custom_time_25</v>
       </c>
     </row>
-    <row r="257" spans="1:11" ht="31.5" thickBot="1">
+    <row r="257" spans="1:11" ht="31.2" thickBot="1">
       <c r="A257" s="4" t="s">
         <v>307</v>
       </c>
@@ -18984,7 +18992,7 @@
         <v>TS-UD-COH-SCR-002test_011_weights_per_project_type</v>
       </c>
     </row>
-    <row r="258" spans="1:11" ht="31.5" thickBot="1">
+    <row r="258" spans="1:11" ht="31.2" thickBot="1">
       <c r="A258" s="4" t="s">
         <v>307</v>
       </c>
@@ -19013,7 +19021,7 @@
         <v>TS-UD-COH-SCR-002test_012_weights_history_tracking</v>
       </c>
     </row>
-    <row r="259" spans="1:11" ht="31.5" thickBot="1">
+    <row r="259" spans="1:11" ht="31.2" thickBot="1">
       <c r="A259" s="4" t="s">
         <v>321</v>
       </c>
@@ -19030,7 +19038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="260" spans="1:11" ht="31.5" thickBot="1">
+    <row r="260" spans="1:11" ht="31.2" thickBot="1">
       <c r="A260" s="4" t="s">
         <v>322</v>
       </c>
@@ -19059,7 +19067,7 @@
         <v>TS-UD-COH-GAM-001test_001_detect_mass_changes_15_in_30min</v>
       </c>
     </row>
-    <row r="261" spans="1:11" ht="31.5" thickBot="1">
+    <row r="261" spans="1:11" ht="31.2" thickBot="1">
       <c r="A261" s="4" t="s">
         <v>322</v>
       </c>
@@ -19088,7 +19096,7 @@
         <v>TS-UD-COH-GAM-001test_002_no_violation_10_in_60min</v>
       </c>
     </row>
-    <row r="262" spans="1:11" ht="31.5" thickBot="1">
+    <row r="262" spans="1:11" ht="31.2" thickBot="1">
       <c r="A262" s="4" t="s">
         <v>322</v>
       </c>
@@ -19117,7 +19125,7 @@
         <v>TS-UD-COH-GAM-001test_003_mass_changes_window_sliding</v>
       </c>
     </row>
-    <row r="263" spans="1:11" ht="31.5" thickBot="1">
+    <row r="263" spans="1:11" ht="31.2" thickBot="1">
       <c r="A263" s="4" t="s">
         <v>322</v>
       </c>
@@ -19146,7 +19154,7 @@
         <v>TS-UD-COH-GAM-001test_004_mass_changes_flag_for_review</v>
       </c>
     </row>
-    <row r="264" spans="1:11" ht="31.5" thickBot="1">
+    <row r="264" spans="1:11" ht="31.2" thickBot="1">
       <c r="A264" s="4" t="s">
         <v>322</v>
       </c>
@@ -19175,7 +19183,7 @@
         <v>TS-UD-COH-GAM-001test_005_detect_resolve_reintroduce_4_times</v>
       </c>
     </row>
-    <row r="265" spans="1:11" ht="31.5" thickBot="1">
+    <row r="265" spans="1:11" ht="31.2" thickBot="1">
       <c r="A265" s="4" t="s">
         <v>322</v>
       </c>
@@ -19204,7 +19212,7 @@
         <v>TS-UD-COH-GAM-001test_006_no_violation_2_times</v>
       </c>
     </row>
-    <row r="266" spans="1:11" ht="31.5" thickBot="1">
+    <row r="266" spans="1:11" ht="31.2" thickBot="1">
       <c r="A266" s="4" t="s">
         <v>322</v>
       </c>
@@ -19233,7 +19241,7 @@
         <v>TS-UD-COH-GAM-001test_007_hash_comparison_same_content</v>
       </c>
     </row>
-    <row r="267" spans="1:11" ht="31.5" thickBot="1">
+    <row r="267" spans="1:11" ht="31.2" thickBot="1">
       <c r="A267" s="4" t="s">
         <v>322</v>
       </c>
@@ -19262,7 +19270,7 @@
         <v>TS-UD-COH-GAM-001test_008_penalty_minus_5_points</v>
       </c>
     </row>
-    <row r="268" spans="1:11" ht="31.5" thickBot="1">
+    <row r="268" spans="1:11" ht="31.2" thickBot="1">
       <c r="A268" s="4" t="s">
         <v>322</v>
       </c>
@@ -19291,7 +19299,7 @@
         <v>TS-UD-COH-GAM-001test_009_detect_95_percent_3_docs</v>
       </c>
     </row>
-    <row r="269" spans="1:11" ht="31.5" thickBot="1">
+    <row r="269" spans="1:11" ht="31.2" thickBot="1">
       <c r="A269" s="4" t="s">
         <v>322</v>
       </c>
@@ -19320,7 +19328,7 @@
         <v>TS-UD-COH-GAM-001test_010_no_violation_95_percent_50_docs</v>
       </c>
     </row>
-    <row r="270" spans="1:11" ht="31.5" thickBot="1">
+    <row r="270" spans="1:11" ht="31.2" thickBot="1">
       <c r="A270" s="4" t="s">
         <v>322</v>
       </c>
@@ -19349,7 +19357,7 @@
         <v>TS-UD-COH-GAM-001test_011_threshold_90_percent_5_docs</v>
       </c>
     </row>
-    <row r="271" spans="1:11" ht="31.5" thickBot="1">
+    <row r="271" spans="1:11" ht="31.2" thickBot="1">
       <c r="A271" s="4" t="s">
         <v>322</v>
       </c>
@@ -19378,7 +19386,7 @@
         <v>TS-UD-COH-GAM-001test_012_require_audit_action</v>
       </c>
     </row>
-    <row r="272" spans="1:11" ht="31.5" thickBot="1">
+    <row r="272" spans="1:11" ht="31.2" thickBot="1">
       <c r="A272" s="4" t="s">
         <v>322</v>
       </c>
@@ -19407,7 +19415,7 @@
         <v>TS-UD-COH-GAM-001test_013_detect_weight_change_25_percent</v>
       </c>
     </row>
-    <row r="273" spans="1:11" ht="31.5" thickBot="1">
+    <row r="273" spans="1:11" ht="31.2" thickBot="1">
       <c r="A273" s="4" t="s">
         <v>322</v>
       </c>
@@ -19436,7 +19444,7 @@
         <v>TS-UD-COH-GAM-001test_014_no_violation_change_15_percent</v>
       </c>
     </row>
-    <row r="274" spans="1:11" ht="31.5" thickBot="1">
+    <row r="274" spans="1:11" ht="31.2" thickBot="1">
       <c r="A274" s="4" t="s">
         <v>322</v>
       </c>
@@ -19465,7 +19473,7 @@
         <v>TS-UD-COH-GAM-001test_015_24h_window_tracking</v>
       </c>
     </row>
-    <row r="275" spans="1:11" ht="31.5" thickBot="1">
+    <row r="275" spans="1:11" ht="31.2" thickBot="1">
       <c r="A275" s="4" t="s">
         <v>322</v>
       </c>
@@ -19494,7 +19502,7 @@
         <v>TS-UD-COH-GAM-001test_016_notify_admin_action</v>
       </c>
     </row>
-    <row r="276" spans="1:11" ht="31.5" thickBot="1">
+    <row r="276" spans="1:11" ht="31.2" thickBot="1">
       <c r="A276" s="4" t="s">
         <v>340</v>
       </c>
@@ -19515,7 +19523,7 @@
         <v>TS-UD-COH-ALR-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="277" spans="1:11" ht="31.5" thickBot="1">
+    <row r="277" spans="1:11" ht="31.2" thickBot="1">
       <c r="A277" s="4" t="s">
         <v>341</v>
       </c>
@@ -19547,7 +19555,7 @@
         <v>TS-UD-PRJ-WBS-001test_001_wbs_item_creation_all_fields</v>
       </c>
     </row>
-    <row r="278" spans="1:11" ht="31.5" thickBot="1">
+    <row r="278" spans="1:11" ht="31.2" thickBot="1">
       <c r="A278" s="4" t="s">
         <v>341</v>
       </c>
@@ -19576,7 +19584,7 @@
         <v>TS-UD-PRJ-WBS-001test_002_wbs_item_creation_minimum_fields</v>
       </c>
     </row>
-    <row r="279" spans="1:11" ht="31.5" thickBot="1">
+    <row r="279" spans="1:11" ht="31.2" thickBot="1">
       <c r="A279" s="4" t="s">
         <v>341</v>
       </c>
@@ -19605,7 +19613,7 @@
         <v>TS-UD-PRJ-WBS-001test_003_wbs_item_fails_without_code</v>
       </c>
     </row>
-    <row r="280" spans="1:11" ht="31.5" thickBot="1">
+    <row r="280" spans="1:11" ht="31.2" thickBot="1">
       <c r="A280" s="4" t="s">
         <v>341</v>
       </c>
@@ -19634,7 +19642,7 @@
         <v>TS-UD-PRJ-WBS-001test_004_wbs_item_fails_without_name</v>
       </c>
     </row>
-    <row r="281" spans="1:11" ht="31.5" thickBot="1">
+    <row r="281" spans="1:11" ht="31.2" thickBot="1">
       <c r="A281" s="4" t="s">
         <v>341</v>
       </c>
@@ -19663,7 +19671,7 @@
         <v>TS-UD-PRJ-WBS-001test_005_wbs_item_fails_invalid_level</v>
       </c>
     </row>
-    <row r="282" spans="1:11" ht="31.5" thickBot="1">
+    <row r="282" spans="1:11" ht="31.2" thickBot="1">
       <c r="A282" s="4" t="s">
         <v>341</v>
       </c>
@@ -19692,7 +19700,7 @@
         <v>TS-UD-PRJ-WBS-001test_006_wbs_item_immutability</v>
       </c>
     </row>
-    <row r="283" spans="1:11" ht="31.5" thickBot="1">
+    <row r="283" spans="1:11" ht="31.2" thickBot="1">
       <c r="A283" s="4" t="s">
         <v>341</v>
       </c>
@@ -19721,7 +19729,7 @@
         <v>TS-UD-PRJ-WBS-001test_007_wbs_code_format_1</v>
       </c>
     </row>
-    <row r="284" spans="1:11" ht="31.5" thickBot="1">
+    <row r="284" spans="1:11" ht="31.2" thickBot="1">
       <c r="A284" s="4" t="s">
         <v>341</v>
       </c>
@@ -19750,7 +19758,7 @@
         <v>TS-UD-PRJ-WBS-001test_008_wbs_code_format_1_1</v>
       </c>
     </row>
-    <row r="285" spans="1:11" ht="31.5" thickBot="1">
+    <row r="285" spans="1:11" ht="31.2" thickBot="1">
       <c r="A285" s="4" t="s">
         <v>341</v>
       </c>
@@ -19779,7 +19787,7 @@
         <v>TS-UD-PRJ-WBS-001test_009_wbs_code_format_1_1_1</v>
       </c>
     </row>
-    <row r="286" spans="1:11" ht="31.5" thickBot="1">
+    <row r="286" spans="1:11" ht="31.2" thickBot="1">
       <c r="A286" s="4" t="s">
         <v>341</v>
       </c>
@@ -19808,7 +19816,7 @@
         <v>TS-UD-PRJ-WBS-001test_010_wbs_code_format_1_1_1_1</v>
       </c>
     </row>
-    <row r="287" spans="1:11" ht="31.5" thickBot="1">
+    <row r="287" spans="1:11" ht="31.2" thickBot="1">
       <c r="A287" s="4" t="s">
         <v>341</v>
       </c>
@@ -19837,7 +19845,7 @@
         <v>TS-UD-PRJ-WBS-001test_011_wbs_code_invalid_format_rejected</v>
       </c>
     </row>
-    <row r="288" spans="1:11" ht="31.5" thickBot="1">
+    <row r="288" spans="1:11" ht="31.2" thickBot="1">
       <c r="A288" s="4" t="s">
         <v>341</v>
       </c>
@@ -19866,7 +19874,7 @@
         <v>TS-UD-PRJ-WBS-001test_012_wbs_code_uniqueness_per_project</v>
       </c>
     </row>
-    <row r="289" spans="1:11" ht="31.5" thickBot="1">
+    <row r="289" spans="1:11" ht="31.2" thickBot="1">
       <c r="A289" s="4" t="s">
         <v>341</v>
       </c>
@@ -19895,7 +19903,7 @@
         <v>TS-UD-PRJ-WBS-001test_013_wbs_level_1_valid</v>
       </c>
     </row>
-    <row r="290" spans="1:11" ht="31.5" thickBot="1">
+    <row r="290" spans="1:11" ht="31.2" thickBot="1">
       <c r="A290" s="4" t="s">
         <v>341</v>
       </c>
@@ -19924,7 +19932,7 @@
         <v>TS-UD-PRJ-WBS-001test_014_wbs_level_4_valid</v>
       </c>
     </row>
-    <row r="291" spans="1:11" ht="31.5" thickBot="1">
+    <row r="291" spans="1:11" ht="31.2" thickBot="1">
       <c r="A291" s="4" t="s">
         <v>341</v>
       </c>
@@ -19953,7 +19961,7 @@
         <v>TS-UD-PRJ-WBS-001test_015_wbs_level_0_invalid</v>
       </c>
     </row>
-    <row r="292" spans="1:11" ht="31.5" thickBot="1">
+    <row r="292" spans="1:11" ht="31.2" thickBot="1">
       <c r="A292" s="4" t="s">
         <v>341</v>
       </c>
@@ -19982,7 +19990,7 @@
         <v>TS-UD-PRJ-WBS-001test_016_wbs_level_5_invalid</v>
       </c>
     </row>
-    <row r="293" spans="1:11" ht="31.5" thickBot="1">
+    <row r="293" spans="1:11" ht="31.2" thickBot="1">
       <c r="A293" s="4" t="s">
         <v>341</v>
       </c>
@@ -20011,7 +20019,7 @@
         <v>TS-UD-PRJ-WBS-001test_017_wbs_level_matches_code_depth</v>
       </c>
     </row>
-    <row r="294" spans="1:11" ht="31.5" thickBot="1">
+    <row r="294" spans="1:11" ht="31.2" thickBot="1">
       <c r="A294" s="4" t="s">
         <v>341</v>
       </c>
@@ -20040,7 +20048,7 @@
         <v>TS-UD-PRJ-WBS-001test_018_wbs_level_parent_child_validation</v>
       </c>
     </row>
-    <row r="295" spans="1:11" ht="31.5" thickBot="1">
+    <row r="295" spans="1:11" ht="31.2" thickBot="1">
       <c r="A295" s="4" t="s">
         <v>363</v>
       </c>
@@ -20061,7 +20069,7 @@
         <v>TS-UD-PRJ-WBS-002Tests not individually listed</v>
       </c>
     </row>
-    <row r="296" spans="1:11" ht="31.5" thickBot="1">
+    <row r="296" spans="1:11" ht="31.2" thickBot="1">
       <c r="A296" s="4" t="s">
         <v>364</v>
       </c>
@@ -20082,7 +20090,7 @@
         <v>TS-UD-PRJ-WBS-003Tests not individually listed</v>
       </c>
     </row>
-    <row r="297" spans="1:11" ht="31.5" thickBot="1">
+    <row r="297" spans="1:11" ht="31.2" thickBot="1">
       <c r="A297" s="4" t="s">
         <v>365</v>
       </c>
@@ -20103,7 +20111,7 @@
         <v>TS-UD-PRJ-WBS-004Tests not individually listed</v>
       </c>
     </row>
-    <row r="298" spans="1:11" ht="31.5" thickBot="1">
+    <row r="298" spans="1:11" ht="31.2" thickBot="1">
       <c r="A298" s="4" t="s">
         <v>366</v>
       </c>
@@ -20124,7 +20132,7 @@
         <v>TS-UD-PRJ-PRJ-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="299" spans="1:11" ht="31.5" thickBot="1">
+    <row r="299" spans="1:11" ht="31.2" thickBot="1">
       <c r="A299" s="4" t="s">
         <v>367</v>
       </c>
@@ -20145,7 +20153,7 @@
         <v>TS-UD-PRJ-DTO-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="300" spans="1:11" ht="46.5" thickBot="1">
+    <row r="300" spans="1:11" ht="31.2" thickBot="1">
       <c r="A300" s="4" t="s">
         <v>368</v>
       </c>
@@ -20166,7 +20174,7 @@
         <v>TS-UD-PROC-BOM-001Tests not individually listed</v>
       </c>
     </row>
-    <row r="301" spans="1:11" ht="46.5" thickBot="1">
+    <row r="301" spans="1:11" ht="31.2" thickBot="1">
       <c r="A301" s="4" t="s">
         <v>370</v>
       </c>
@@ -20187,7 +20195,7 @@
         <v>TS-UD-PROC-BOM-002Tests not individually listed</v>
       </c>
     </row>
-    <row r="302" spans="1:11" ht="46.5" thickBot="1">
+    <row r="302" spans="1:11" ht="31.2" thickBot="1">
       <c r="A302" s="4" t="s">
         <v>371</v>
       </c>
@@ -20219,7 +20227,7 @@
         <v>TS-UD-PROC-LTM-001test_001_optimal_date_production_only</v>
       </c>
     </row>
-    <row r="303" spans="1:11" ht="46.5" thickBot="1">
+    <row r="303" spans="1:11" ht="31.2" thickBot="1">
       <c r="A303" s="4" t="s">
         <v>371</v>
       </c>
@@ -20248,7 +20256,7 @@
         <v>TS-UD-PROC-LTM-001test_002_optimal_date_production_transit</v>
       </c>
     </row>
-    <row r="304" spans="1:11" ht="46.5" thickBot="1">
+    <row r="304" spans="1:11" ht="31.2" thickBot="1">
       <c r="A304" s="4" t="s">
         <v>371</v>
       </c>
@@ -20277,7 +20285,7 @@
         <v>TS-UD-PROC-LTM-001test_003_optimal_date_production_transit_buffer</v>
       </c>
     </row>
-    <row r="305" spans="1:11" ht="46.5" thickBot="1">
+    <row r="305" spans="1:11" ht="31.2" thickBot="1">
       <c r="A305" s="4" t="s">
         <v>371</v>
       </c>
@@ -20306,7 +20314,7 @@
         <v>TS-UD-PROC-LTM-001test_004_optimal_date_all_components</v>
       </c>
     </row>
-    <row r="306" spans="1:11" ht="46.5" thickBot="1">
+    <row r="306" spans="1:11" ht="31.2" thickBot="1">
       <c r="A306" s="4" t="s">
         <v>371</v>
       </c>
@@ -20335,7 +20343,7 @@
         <v>TS-UD-PROC-LTM-001test_005_lead_time_breakdown_returned</v>
       </c>
     </row>
-    <row r="307" spans="1:11" ht="46.5" thickBot="1">
+    <row r="307" spans="1:11" ht="31.2" thickBot="1">
       <c r="A307" s="4" t="s">
         <v>371</v>
       </c>
@@ -20364,7 +20372,7 @@
         <v>TS-UD-PROC-LTM-001test_006_required_on_site_calculation</v>
       </c>
     </row>
-    <row r="308" spans="1:11" ht="46.5" thickBot="1">
+    <row r="308" spans="1:11" ht="31.2" thickBot="1">
       <c r="A308" s="4" t="s">
         <v>371</v>
       </c>
@@ -20393,7 +20401,7 @@
         <v>TS-UD-PROC-LTM-001test_007_business_days_calculation</v>
       </c>
     </row>
-    <row r="309" spans="1:11" ht="46.5" thickBot="1">
+    <row r="309" spans="1:11" ht="31.2" thickBot="1">
       <c r="A309" s="4" t="s">
         <v>371</v>
       </c>
@@ -20422,7 +20430,7 @@
         <v>TS-UD-PROC-LTM-001test_008_weekend_exclusion</v>
       </c>
     </row>
-    <row r="310" spans="1:11" ht="46.5" thickBot="1">
+    <row r="310" spans="1:11" ht="31.2" thickBot="1">
       <c r="A310" s="4" t="s">
         <v>371</v>
       </c>
@@ -20451,7 +20459,7 @@
         <v>TS-UD-PROC-LTM-001test_009_holiday_exclusion</v>
       </c>
     </row>
-    <row r="311" spans="1:11" ht="46.5" thickBot="1">
+    <row r="311" spans="1:11" ht="31.2" thickBot="1">
       <c r="A311" s="4" t="s">
         <v>371</v>
       </c>
@@ -20480,7 +20488,7 @@
         <v>TS-UD-PROC-LTM-001test_010_delivery_on_weekend_adjusted</v>
       </c>
     </row>
-    <row r="312" spans="1:11" ht="46.5" thickBot="1">
+    <row r="312" spans="1:11" ht="31.2" thickBot="1">
       <c r="A312" s="4" t="s">
         <v>371</v>
       </c>
@@ -20509,7 +20517,7 @@
         <v>TS-UD-PROC-LTM-001test_011_mixed_calendar_business_days</v>
       </c>
     </row>
-    <row r="313" spans="1:11" ht="46.5" thickBot="1">
+    <row r="313" spans="1:11" ht="31.2" thickBot="1">
       <c r="A313" s="4" t="s">
         <v>371</v>
       </c>
@@ -20538,7 +20546,7 @@
         <v>TS-UD-PROC-LTM-001test_012_alert_r14_date_passed</v>
       </c>
     </row>
-    <row r="314" spans="1:11" ht="46.5" thickBot="1">
+    <row r="314" spans="1:11" ht="31.2" thickBot="1">
       <c r="A314" s="4" t="s">
         <v>371</v>
       </c>
@@ -20567,7 +20575,7 @@
         <v>TS-UD-PROC-LTM-001test_013_alert_r14_tight_margin_3_days</v>
       </c>
     </row>
-    <row r="315" spans="1:11" ht="46.5" thickBot="1">
+    <row r="315" spans="1:11" ht="31.2" thickBot="1">
       <c r="A315" s="4" t="s">
         <v>371</v>
       </c>
@@ -20596,7 +20604,7 @@
         <v>TS-UD-PROC-LTM-001test_014_alert_severity_critical_passed</v>
       </c>
     </row>
-    <row r="316" spans="1:11" ht="46.5" thickBot="1">
+    <row r="316" spans="1:11" ht="31.2" thickBot="1">
       <c r="A316" s="4" t="s">
         <v>371</v>
       </c>
@@ -20625,7 +20633,7 @@
         <v>TS-UD-PROC-LTM-001test_015_alert_severity_warning_tight</v>
       </c>
     </row>
-    <row r="317" spans="1:11" ht="46.5" thickBot="1">
+    <row r="317" spans="1:11" ht="31.2" thickBot="1">
       <c r="A317" s="4" t="s">
         <v>371</v>
       </c>
@@ -20654,7 +20662,7 @@
         <v>TS-UD-PROC-LTM-001test_016_no_alert_sufficient_margin</v>
       </c>
     </row>
-    <row r="318" spans="1:11" ht="46.5" thickBot="1">
+    <row r="318" spans="1:11" ht="31.2" thickBot="1">
       <c r="A318" s="4" t="s">
         <v>390</v>
       </c>
@@ -20680,7 +20688,7 @@
         <v>TS-UD-PROC-LTM-002test_001_exw_buyer_full_responsibility</v>
       </c>
     </row>
-    <row r="319" spans="1:11" ht="46.5" thickBot="1">
+    <row r="319" spans="1:11" ht="31.2" thickBot="1">
       <c r="A319" s="4" t="s">
         <v>390</v>
       </c>
@@ -20706,7 +20714,7 @@
         <v>TS-UD-PROC-LTM-002test_002_exw_transit_time_included</v>
       </c>
     </row>
-    <row r="320" spans="1:11" ht="46.5" thickBot="1">
+    <row r="320" spans="1:11" ht="31.2" thickBot="1">
       <c r="A320" s="4" t="s">
         <v>390</v>
       </c>
@@ -20732,7 +20740,7 @@
         <v>TS-UD-PROC-LTM-002test_003_exw_customs_included</v>
       </c>
     </row>
-    <row r="321" spans="1:11" ht="46.5" thickBot="1">
+    <row r="321" spans="1:11" ht="31.2" thickBot="1">
       <c r="A321" s="4" t="s">
         <v>390</v>
       </c>
@@ -20758,7 +20766,7 @@
         <v>TS-UD-PROC-LTM-002test_004_fob_shared_responsibility</v>
       </c>
     </row>
-    <row r="322" spans="1:11" ht="46.5" thickBot="1">
+    <row r="322" spans="1:11" ht="31.2" thickBot="1">
       <c r="A322" s="4" t="s">
         <v>390</v>
       </c>
@@ -20784,7 +20792,7 @@
         <v>TS-UD-PROC-LTM-002test_005_fob_port_handover</v>
       </c>
     </row>
-    <row r="323" spans="1:11" ht="46.5" thickBot="1">
+    <row r="323" spans="1:11" ht="31.2" thickBot="1">
       <c r="A323" s="4" t="s">
         <v>390</v>
       </c>
@@ -20810,7 +20818,7 @@
         <v>TS-UD-PROC-LTM-002test_006_fob_insurance_buyer</v>
       </c>
     </row>
-    <row r="324" spans="1:11" ht="46.5" thickBot="1">
+    <row r="324" spans="1:11" ht="31.2" thickBot="1">
       <c r="A324" s="4" t="s">
         <v>390</v>
       </c>
@@ -20836,7 +20844,7 @@
         <v>TS-UD-PROC-LTM-002test_007_cif_seller_insurance</v>
       </c>
     </row>
-    <row r="325" spans="1:11" ht="46.5" thickBot="1">
+    <row r="325" spans="1:11" ht="31.2" thickBot="1">
       <c r="A325" s="4" t="s">
         <v>390</v>
       </c>
@@ -20862,7 +20870,7 @@
         <v>TS-UD-PROC-LTM-002test_008_cif_port_to_port</v>
       </c>
     </row>
-    <row r="326" spans="1:11" ht="46.5" thickBot="1">
+    <row r="326" spans="1:11" ht="31.2" thickBot="1">
       <c r="A326" s="4" t="s">
         <v>390</v>
       </c>
@@ -20888,7 +20896,7 @@
         <v>TS-UD-PROC-LTM-002test_009_cif_customs_buyer</v>
       </c>
     </row>
-    <row r="327" spans="1:11" ht="46.5" thickBot="1">
+    <row r="327" spans="1:11" ht="31.2" thickBot="1">
       <c r="A327" s="4" t="s">
         <v>390</v>
       </c>
@@ -20914,7 +20922,7 @@
         <v>TS-UD-PROC-LTM-002test_010_ddp_seller_full_responsibility</v>
       </c>
     </row>
-    <row r="328" spans="1:11" ht="46.5" thickBot="1">
+    <row r="328" spans="1:11" ht="31.2" thickBot="1">
       <c r="A328" s="4" t="s">
         <v>390</v>
       </c>
@@ -20940,7 +20948,7 @@
         <v>TS-UD-PROC-LTM-002test_011_ddp_no_customs_buyer</v>
       </c>
     </row>
-    <row r="329" spans="1:11" ht="46.5" thickBot="1">
+    <row r="329" spans="1:11" ht="31.2" thickBot="1">
       <c r="A329" s="4" t="s">
         <v>390</v>
       </c>
@@ -20966,7 +20974,7 @@
         <v>TS-UD-PROC-LTM-002test_012_ddp_door_to_door</v>
       </c>
     </row>
-    <row r="330" spans="1:11" ht="46.5" thickBot="1">
+    <row r="330" spans="1:11" ht="31.2" thickBot="1">
       <c r="A330" s="4" t="s">
         <v>390</v>
       </c>
@@ -20992,7 +21000,7 @@
         <v>TS-UD-PROC-LTM-002test_013_incoterm_comparison_same_route</v>
       </c>
     </row>
-    <row r="331" spans="1:11" ht="46.5" thickBot="1">
+    <row r="331" spans="1:11" ht="31.2" thickBot="1">
       <c r="A331" s="4" t="s">
         <v>390</v>
       </c>
@@ -21018,7 +21026,7 @@
         <v>TS-UD-PROC-LTM-002test_014_incoterm_impact_on_lead_time</v>
       </c>
     </row>
-    <row r="332" spans="1:11" ht="46.5" thickBot="1">
+    <row r="332" spans="1:11" ht="31.2" thickBot="1">
       <c r="A332" s="4" t="s">
         <v>406</v>
       </c>
@@ -21035,7 +21043,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="333" spans="1:11" ht="46.5" thickBot="1">
+    <row r="333" spans="1:11" ht="31.2" thickBot="1">
       <c r="A333" s="4" t="s">
         <v>407</v>
       </c>
@@ -21052,7 +21060,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="334" spans="1:11" ht="46.5" thickBot="1">
+    <row r="334" spans="1:11" ht="31.2" thickBot="1">
       <c r="A334" s="4" t="s">
         <v>408</v>
       </c>
@@ -21069,7 +21077,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="335" spans="1:11" ht="46.5" thickBot="1">
+    <row r="335" spans="1:11" ht="31.2" thickBot="1">
       <c r="A335" s="4" t="s">
         <v>409</v>
       </c>
@@ -21086,7 +21094,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="336" spans="1:11" ht="46.5" thickBot="1">
+    <row r="336" spans="1:11" ht="31.2" thickBot="1">
       <c r="A336" s="4" t="s">
         <v>411</v>
       </c>
@@ -21103,7 +21111,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="337" spans="1:10" ht="46.5" thickBot="1">
+    <row r="337" spans="1:10" ht="31.2" thickBot="1">
       <c r="A337" s="4" t="s">
         <v>412</v>
       </c>
@@ -21120,7 +21128,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="338" spans="1:10" ht="46.5" thickBot="1">
+    <row r="338" spans="1:10" ht="31.2" thickBot="1">
       <c r="A338" s="4" t="s">
         <v>413</v>
       </c>
@@ -21136,7 +21144,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="339" spans="1:10" ht="46.5" thickBot="1">
+    <row r="339" spans="1:10" ht="31.2" thickBot="1">
       <c r="A339" s="4" t="s">
         <v>414</v>
       </c>
@@ -21152,7 +21160,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="340" spans="1:10" ht="46.5" thickBot="1">
+    <row r="340" spans="1:10" ht="31.2" thickBot="1">
       <c r="A340" s="4" t="s">
         <v>415</v>
       </c>
@@ -21168,7 +21176,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="341" spans="1:10" ht="46.5" thickBot="1">
+    <row r="341" spans="1:10" ht="31.2" thickBot="1">
       <c r="A341" s="4" t="s">
         <v>416</v>
       </c>
@@ -21184,7 +21192,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="342" spans="1:10" ht="31.5" thickBot="1">
+    <row r="342" spans="1:10" ht="31.2" thickBot="1">
       <c r="A342" s="4" t="s">
         <v>417</v>
       </c>
@@ -21200,7 +21208,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="343" spans="1:10" ht="31.5" thickBot="1">
+    <row r="343" spans="1:10" ht="31.2" thickBot="1">
       <c r="A343" s="4" t="s">
         <v>419</v>
       </c>
@@ -21216,7 +21224,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="344" spans="1:10" ht="31.5" thickBot="1">
+    <row r="344" spans="1:10" ht="31.2" thickBot="1">
       <c r="A344" s="4" t="s">
         <v>420</v>
       </c>
@@ -21232,7 +21240,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="345" spans="1:10" ht="31.5" thickBot="1">
+    <row r="345" spans="1:10" ht="31.2" thickBot="1">
       <c r="A345" s="4" t="s">
         <v>421</v>
       </c>
@@ -21248,7 +21256,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="346" spans="1:10" ht="31.5" thickBot="1">
+    <row r="346" spans="1:10" ht="31.2" thickBot="1">
       <c r="A346" s="4" t="s">
         <v>422</v>
       </c>
@@ -21264,7 +21272,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="347" spans="1:10" ht="31.5" thickBot="1">
+    <row r="347" spans="1:10" ht="31.2" thickBot="1">
       <c r="A347" s="4" t="s">
         <v>423</v>
       </c>
@@ -21280,7 +21288,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="348" spans="1:10" ht="31.5" thickBot="1">
+    <row r="348" spans="1:10" ht="31.2" thickBot="1">
       <c r="A348" s="4" t="s">
         <v>425</v>
       </c>
@@ -21296,7 +21304,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="349" spans="1:10" ht="31.5" thickBot="1">
+    <row r="349" spans="1:10" ht="31.2" thickBot="1">
       <c r="A349" s="4" t="s">
         <v>426</v>
       </c>
@@ -21312,7 +21320,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="350" spans="1:10" ht="31.5" thickBot="1">
+    <row r="350" spans="1:10" ht="31.2" thickBot="1">
       <c r="A350" s="4" t="s">
         <v>427</v>
       </c>
@@ -21328,7 +21336,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="351" spans="1:10" ht="31.5" thickBot="1">
+    <row r="351" spans="1:10" ht="31.2" thickBot="1">
       <c r="A351" s="4" t="s">
         <v>428</v>
       </c>
@@ -21344,7 +21352,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="352" spans="1:10" ht="31.5" thickBot="1">
+    <row r="352" spans="1:10" ht="31.2" thickBot="1">
       <c r="A352" s="10" t="s">
         <v>429</v>
       </c>
@@ -21363,7 +21371,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="353" spans="1:10" ht="31.5" thickBot="1">
+    <row r="353" spans="1:10" ht="31.2" thickBot="1">
       <c r="A353" s="10" t="s">
         <v>430</v>
       </c>
@@ -21382,7 +21390,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="354" spans="1:10" ht="31.5" thickBot="1">
+    <row r="354" spans="1:10" ht="31.2" thickBot="1">
       <c r="A354" s="4" t="s">
         <v>431</v>
       </c>
@@ -21398,7 +21406,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="355" spans="1:10" ht="31.5" thickBot="1">
+    <row r="355" spans="1:10" ht="31.2" thickBot="1">
       <c r="A355" s="4" t="s">
         <v>432</v>
       </c>
@@ -21414,7 +21422,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="356" spans="1:10" ht="31.5" thickBot="1">
+    <row r="356" spans="1:10" ht="31.2" thickBot="1">
       <c r="A356" s="4" t="s">
         <v>433</v>
       </c>
@@ -21430,7 +21438,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="357" spans="1:10" ht="31.5" thickBot="1">
+    <row r="357" spans="1:10" ht="31.2" thickBot="1">
       <c r="A357" s="4" t="s">
         <v>434</v>
       </c>
@@ -21446,7 +21454,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="358" spans="1:10" ht="31.5" thickBot="1">
+    <row r="358" spans="1:10" ht="31.2" thickBot="1">
       <c r="A358" s="4" t="s">
         <v>435</v>
       </c>
@@ -21462,7 +21470,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="359" spans="1:10" ht="31.5" thickBot="1">
+    <row r="359" spans="1:10" ht="31.2" thickBot="1">
       <c r="A359" s="4" t="s">
         <v>436</v>
       </c>
@@ -21478,7 +21486,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="360" spans="1:10" ht="31.5" thickBot="1">
+    <row r="360" spans="1:10" ht="31.2" thickBot="1">
       <c r="A360" s="4" t="s">
         <v>437</v>
       </c>
@@ -21494,7 +21502,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="361" spans="1:10" ht="31.5" thickBot="1">
+    <row r="361" spans="1:10" ht="31.2" thickBot="1">
       <c r="A361" s="4" t="s">
         <v>438</v>
       </c>
@@ -21510,7 +21518,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="362" spans="1:10" ht="31.5" thickBot="1">
+    <row r="362" spans="1:10" ht="31.2" thickBot="1">
       <c r="A362" s="4" t="s">
         <v>439</v>
       </c>
@@ -21526,7 +21534,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="363" spans="1:10" ht="31.5" thickBot="1">
+    <row r="363" spans="1:10" ht="31.2" thickBot="1">
       <c r="A363" s="4" t="s">
         <v>441</v>
       </c>
@@ -21542,7 +21550,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="364" spans="1:10" ht="31.5" thickBot="1">
+    <row r="364" spans="1:10" ht="31.2" thickBot="1">
       <c r="A364" s="4" t="s">
         <v>442</v>
       </c>
@@ -21558,7 +21566,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="365" spans="1:10" ht="31.5" thickBot="1">
+    <row r="365" spans="1:10" ht="31.2" thickBot="1">
       <c r="A365" s="4" t="s">
         <v>443</v>
       </c>
@@ -21574,7 +21582,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="366" spans="1:10" ht="31.5" thickBot="1">
+    <row r="366" spans="1:10" ht="31.2" thickBot="1">
       <c r="A366" s="4" t="s">
         <v>444</v>
       </c>
@@ -21590,7 +21598,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="367" spans="1:10" ht="31.5" thickBot="1">
+    <row r="367" spans="1:10" ht="31.2" thickBot="1">
       <c r="A367" s="4" t="s">
         <v>445</v>
       </c>
@@ -21606,7 +21614,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="368" spans="1:10" ht="31.5" thickBot="1">
+    <row r="368" spans="1:10" ht="31.2" thickBot="1">
       <c r="A368" s="4" t="s">
         <v>446</v>
       </c>
@@ -21622,7 +21630,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="369" spans="1:10" ht="31.5" thickBot="1">
+    <row r="369" spans="1:10" ht="31.2" thickBot="1">
       <c r="A369" s="4" t="s">
         <v>447</v>
       </c>
@@ -21641,7 +21649,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="370" spans="1:10" ht="31.5" thickBot="1">
+    <row r="370" spans="1:10" ht="31.2" thickBot="1">
       <c r="A370" s="4" t="s">
         <v>450</v>
       </c>
@@ -21660,7 +21668,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="371" spans="1:10" ht="31.5" thickBot="1">
+    <row r="371" spans="1:10" ht="31.2" thickBot="1">
       <c r="A371" s="4" t="s">
         <v>451</v>
       </c>
@@ -21676,7 +21684,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="372" spans="1:10" ht="31.5" thickBot="1">
+    <row r="372" spans="1:10" ht="31.2" thickBot="1">
       <c r="A372" s="4" t="s">
         <v>453</v>
       </c>
@@ -21692,7 +21700,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="373" spans="1:10" ht="31.5" thickBot="1">
+    <row r="373" spans="1:10" ht="31.2" thickBot="1">
       <c r="A373" s="4" t="s">
         <v>454</v>
       </c>
@@ -21711,7 +21719,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="374" spans="1:10" ht="31.5" thickBot="1">
+    <row r="374" spans="1:10" ht="31.2" thickBot="1">
       <c r="A374" s="4" t="s">
         <v>455</v>
       </c>
@@ -21727,7 +21735,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="375" spans="1:10" ht="31.5" thickBot="1">
+    <row r="375" spans="1:10" ht="31.2" thickBot="1">
       <c r="A375" s="4" t="s">
         <v>457</v>
       </c>
@@ -21743,7 +21751,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="376" spans="1:10" ht="31.5" thickBot="1">
+    <row r="376" spans="1:10" ht="31.2" thickBot="1">
       <c r="A376" s="4" t="s">
         <v>458</v>
       </c>
@@ -21759,7 +21767,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="377" spans="1:10" ht="31.5" thickBot="1">
+    <row r="377" spans="1:10" ht="31.2" thickBot="1">
       <c r="A377" s="4" t="s">
         <v>459</v>
       </c>
@@ -21775,7 +21783,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="378" spans="1:10" ht="16.5" thickBot="1">
+    <row r="378" spans="1:10" ht="16.2" thickBot="1">
       <c r="A378" s="12" t="s">
         <v>460</v>
       </c>
@@ -21794,7 +21802,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="379" spans="1:10" ht="16.5" thickBot="1">
+    <row r="379" spans="1:10" ht="16.2" thickBot="1">
       <c r="A379" s="4" t="s">
         <v>462</v>
       </c>
@@ -21813,7 +21821,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="380" spans="1:10" ht="16.5" thickBot="1">
+    <row r="380" spans="1:10" ht="16.2" thickBot="1">
       <c r="A380" s="4" t="s">
         <v>463</v>
       </c>
@@ -21832,7 +21840,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="381" spans="1:10" ht="16.5" thickBot="1">
+    <row r="381" spans="1:10" ht="16.2" thickBot="1">
       <c r="A381" s="4" t="s">
         <v>464</v>
       </c>
@@ -21848,7 +21856,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="382" spans="1:10" ht="16.5" thickBot="1">
+    <row r="382" spans="1:10" ht="16.2" thickBot="1">
       <c r="A382" s="4" t="s">
         <v>465</v>
       </c>
@@ -21864,7 +21872,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="383" spans="1:10" ht="16.5" thickBot="1">
+    <row r="383" spans="1:10" ht="16.2" thickBot="1">
       <c r="A383" s="4" t="s">
         <v>466</v>
       </c>
@@ -21880,7 +21888,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="384" spans="1:10" ht="16.5" thickBot="1">
+    <row r="384" spans="1:10" ht="16.2" thickBot="1">
       <c r="A384" s="4" t="s">
         <v>467</v>
       </c>
@@ -21896,7 +21904,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="385" spans="1:10" ht="16.5" thickBot="1">
+    <row r="385" spans="1:10" ht="16.2" thickBot="1">
       <c r="A385" s="4" t="s">
         <v>468</v>
       </c>
@@ -21912,7 +21920,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="386" spans="1:10" ht="16.5" thickBot="1">
+    <row r="386" spans="1:10" ht="16.2" thickBot="1">
       <c r="A386" s="4" t="s">
         <v>469</v>
       </c>
@@ -21928,7 +21936,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="387" spans="1:10" ht="16.5" thickBot="1">
+    <row r="387" spans="1:10" ht="16.2" thickBot="1">
       <c r="A387" s="4" t="s">
         <v>470</v>
       </c>
@@ -21944,7 +21952,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="388" spans="1:10" ht="16.5" thickBot="1">
+    <row r="388" spans="1:10" ht="16.2" thickBot="1">
       <c r="A388" s="4" t="s">
         <v>471</v>
       </c>
@@ -21960,7 +21968,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="389" spans="1:10" ht="16.5" thickBot="1">
+    <row r="389" spans="1:10" ht="16.2" thickBot="1">
       <c r="A389" s="4" t="s">
         <v>472</v>
       </c>
@@ -21976,7 +21984,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="390" spans="1:10" ht="16.5" thickBot="1">
+    <row r="390" spans="1:10" ht="16.2" thickBot="1">
       <c r="A390" s="4" t="s">
         <v>473</v>
       </c>
@@ -21992,7 +22000,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="391" spans="1:10" ht="16.5" thickBot="1">
+    <row r="391" spans="1:10" ht="16.2" thickBot="1">
       <c r="A391" s="4" t="s">
         <v>474</v>
       </c>
@@ -22011,7 +22019,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="392" spans="1:10" ht="16.5" thickBot="1">
+    <row r="392" spans="1:10" ht="16.2" thickBot="1">
       <c r="A392" s="4" t="s">
         <v>475</v>
       </c>
@@ -22030,7 +22038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="393" spans="1:10" ht="16.5" thickBot="1">
+    <row r="393" spans="1:10" ht="16.2" thickBot="1">
       <c r="A393" s="4" t="s">
         <v>476</v>
       </c>
@@ -22049,7 +22057,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="394" spans="1:10" ht="16.5" thickBot="1">
+    <row r="394" spans="1:10" ht="16.2" thickBot="1">
       <c r="A394" s="4" t="s">
         <v>477</v>
       </c>
@@ -22065,7 +22073,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="395" spans="1:10" ht="16.5" thickBot="1">
+    <row r="395" spans="1:10" ht="16.2" thickBot="1">
       <c r="A395" s="4" t="s">
         <v>479</v>
       </c>
@@ -22081,7 +22089,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="396" spans="1:10" ht="16.5" thickBot="1">
+    <row r="396" spans="1:10" ht="16.2" thickBot="1">
       <c r="A396" s="4" t="s">
         <v>480</v>
       </c>
@@ -22097,7 +22105,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="397" spans="1:10" ht="16.5" thickBot="1">
+    <row r="397" spans="1:10" ht="16.2" thickBot="1">
       <c r="A397" s="13" t="s">
         <v>481</v>
       </c>
@@ -22119,7 +22127,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="398" spans="1:10" ht="16.5" thickBot="1">
+    <row r="398" spans="1:10" ht="16.2" thickBot="1">
       <c r="A398" s="4" t="s">
         <v>483</v>
       </c>
@@ -22135,7 +22143,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="399" spans="1:10" ht="16.5" thickBot="1">
+    <row r="399" spans="1:10" ht="16.2" thickBot="1">
       <c r="A399" s="4" t="s">
         <v>484</v>
       </c>
@@ -22151,7 +22159,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="400" spans="1:10" ht="16.5" thickBot="1">
+    <row r="400" spans="1:10" ht="16.2" thickBot="1">
       <c r="A400" s="4" t="s">
         <v>485</v>
       </c>
@@ -22167,7 +22175,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="401" spans="1:6" ht="16.5" thickBot="1">
+    <row r="401" spans="1:6" ht="16.2" thickBot="1">
       <c r="A401" s="4" t="s">
         <v>486</v>
       </c>
@@ -22183,7 +22191,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="402" spans="1:6" ht="16.5" thickBot="1">
+    <row r="402" spans="1:6" ht="16.2" thickBot="1">
       <c r="A402" s="4" t="s">
         <v>487</v>
       </c>
@@ -22199,7 +22207,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="403" spans="1:6" ht="15.75" thickBot="1">
+    <row r="403" spans="1:6" ht="15" thickBot="1">
       <c r="A403" s="2"/>
       <c r="B403" s="2"/>
       <c r="C403" s="2"/>
@@ -22207,7 +22215,7 @@
       <c r="E403" s="2"/>
       <c r="F403" s="2"/>
     </row>
-    <row r="404" spans="1:6" ht="15.75" thickBot="1">
+    <row r="404" spans="1:6" ht="15" thickBot="1">
       <c r="A404" s="2"/>
       <c r="B404" s="2"/>
       <c r="C404" s="2"/>
@@ -22223,17 +22231,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8EE910-8E6F-404B-BA4D-060668BC2CAF}">
   <dimension ref="A1:M151"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="26"/>
+    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" style="26"/>
     <col min="7" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="48" thickBot="1">
+    <row r="1" spans="1:12" ht="31.8" thickBot="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -22628,7 +22636,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13.9" customHeight="1">
+    <row r="20" spans="1:13" ht="13.95" customHeight="1">
       <c r="A20" s="31">
         <v>19</v>
       </c>
@@ -22789,7 +22797,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="15.75">
+    <row r="27" spans="1:13" ht="15.6">
       <c r="A27" s="31">
         <v>26</v>
       </c>
@@ -22836,7 +22844,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="45.75">
+    <row r="29" spans="1:13" ht="45.6">
       <c r="A29" s="31">
         <v>28</v>
       </c>
@@ -23133,7 +23141,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="42" spans="1:12" ht="15.75" thickBot="1">
+    <row r="42" spans="1:12" ht="15" thickBot="1">
       <c r="A42" s="31">
         <v>41</v>
       </c>
@@ -23156,7 +23164,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="16.5" thickBot="1">
+    <row r="43" spans="1:12" ht="16.2" thickBot="1">
       <c r="A43" s="31">
         <v>42</v>
       </c>
@@ -23179,7 +23187,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="44" spans="1:12" ht="16.5" thickBot="1">
+    <row r="44" spans="1:12" ht="16.2" thickBot="1">
       <c r="A44" s="31">
         <v>42</v>
       </c>
@@ -23865,7 +23873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:12" ht="15.75" thickBot="1">
+    <row r="75" spans="1:12" ht="15" thickBot="1">
       <c r="A75" s="31">
         <v>71</v>
       </c>
@@ -23888,7 +23896,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="16.5" thickBot="1">
+    <row r="76" spans="1:12" ht="16.2" thickBot="1">
       <c r="A76" s="31">
         <v>72</v>
       </c>
@@ -23911,7 +23919,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="16.5" thickBot="1">
+    <row r="77" spans="1:12" ht="16.2" thickBot="1">
       <c r="A77" s="31">
         <v>73</v>
       </c>
@@ -24224,7 +24232,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="94" spans="1:12" ht="15.75" thickBot="1">
+    <row r="94" spans="1:12" ht="15" thickBot="1">
       <c r="A94" s="31">
         <v>89</v>
       </c>
@@ -24247,7 +24255,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:12" ht="16.899999999999999" customHeight="1" thickBot="1">
+    <row r="95" spans="1:12" ht="16.95" customHeight="1" thickBot="1">
       <c r="A95" s="31">
         <v>72</v>
       </c>
@@ -24310,7 +24318,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="98" spans="1:13" ht="15.75" thickBot="1">
+    <row r="98" spans="1:13" ht="15" thickBot="1">
       <c r="A98" s="31"/>
       <c r="B98" s="18" t="s">
         <v>468</v>
@@ -24329,7 +24337,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:13" ht="16.5" thickBot="1">
+    <row r="99" spans="1:13" ht="16.2" thickBot="1">
       <c r="A99" s="31">
         <v>92</v>
       </c>
@@ -24352,7 +24360,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:13" ht="16.5" thickBot="1">
+    <row r="100" spans="1:13" ht="16.2" thickBot="1">
       <c r="A100" s="31">
         <v>92</v>
       </c>
@@ -24375,7 +24383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:13" ht="16.5" thickBot="1">
+    <row r="101" spans="1:13" ht="16.2" thickBot="1">
       <c r="A101" s="31">
         <v>92</v>
       </c>
@@ -24398,7 +24406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:13" ht="16.5" thickBot="1">
+    <row r="102" spans="1:13" ht="16.2" thickBot="1">
       <c r="A102" s="31">
         <v>92</v>
       </c>
@@ -24419,7 +24427,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="103" spans="1:13" ht="15.75" thickBot="1">
+    <row r="103" spans="1:13" ht="15" thickBot="1">
       <c r="A103" s="31">
         <v>92</v>
       </c>
@@ -24437,7 +24445,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="104" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A104" s="31">
         <v>93</v>
       </c>
@@ -24465,7 +24473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="105" spans="1:13" ht="19.2" customHeight="1">
       <c r="A105" s="32">
         <v>583</v>
       </c>
@@ -24494,7 +24502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="106" spans="1:13" ht="19.2" customHeight="1">
       <c r="A106" s="32">
         <v>584</v>
       </c>
@@ -24520,7 +24528,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="107" spans="1:13" ht="19.2" customHeight="1">
       <c r="A107" s="32">
         <v>585</v>
       </c>
@@ -24544,7 +24552,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="108" spans="1:13" ht="19.2" customHeight="1">
       <c r="A108" s="32">
         <v>586</v>
       </c>
@@ -24568,7 +24576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="109" spans="1:13" ht="19.2" customHeight="1">
       <c r="A109" s="32">
         <v>588</v>
       </c>
@@ -24592,7 +24600,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="110" spans="1:13" ht="19.2" customHeight="1">
       <c r="A110" s="32">
         <v>589</v>
       </c>
@@ -24616,7 +24624,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="111" spans="1:13" ht="19.2" customHeight="1">
       <c r="A111" s="32">
         <v>590</v>
       </c>
@@ -24640,7 +24648,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="112" spans="1:13" ht="19.2" customHeight="1">
       <c r="A112" s="32">
         <v>591</v>
       </c>
@@ -24664,7 +24672,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="113" spans="1:13" ht="19.2" customHeight="1">
       <c r="A113" s="32">
         <v>592</v>
       </c>
@@ -24690,7 +24698,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="114" spans="1:13" ht="19.2" customHeight="1">
       <c r="A114" s="32">
         <v>593</v>
       </c>
@@ -24716,7 +24724,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="115" spans="1:13" ht="19.2" customHeight="1">
       <c r="A115" s="32">
         <v>610</v>
       </c>
@@ -24742,7 +24750,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="116" spans="1:13" ht="19.2" customHeight="1">
       <c r="A116" s="32">
         <v>614</v>
       </c>
@@ -24771,7 +24779,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:13" ht="19.149999999999999" customHeight="1">
+    <row r="117" spans="1:13" ht="19.2" customHeight="1">
       <c r="A117" s="32">
         <v>615</v>
       </c>
@@ -24800,7 +24808,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="118" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A118" s="32">
         <v>616</v>
       </c>
@@ -24829,7 +24837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="119" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A119" s="31">
         <v>94</v>
       </c>
@@ -24850,7 +24858,7 @@
       <c r="J119" s="22"/>
       <c r="K119" s="22"/>
     </row>
-    <row r="120" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="120" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A120" s="31">
         <v>95</v>
       </c>
@@ -24878,7 +24886,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="121" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A121" s="31">
         <v>96</v>
       </c>
@@ -24906,7 +24914,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="122" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A122" s="31">
         <v>97</v>
       </c>
@@ -24934,7 +24942,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="123" spans="1:13" ht="15.75" thickBot="1">
+    <row r="123" spans="1:13" ht="15" thickBot="1">
       <c r="A123" s="32">
         <v>598</v>
       </c>
@@ -24960,7 +24968,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="124" spans="1:13" ht="15.75" thickBot="1">
+    <row r="124" spans="1:13" ht="15" thickBot="1">
       <c r="A124" s="32">
         <v>599</v>
       </c>
@@ -24986,7 +24994,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="125" spans="1:13" ht="15.75" thickBot="1">
+    <row r="125" spans="1:13" ht="15" thickBot="1">
       <c r="A125" s="32">
         <v>600</v>
       </c>
@@ -25012,7 +25020,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:13" ht="15.75" thickBot="1">
+    <row r="126" spans="1:13" ht="15" thickBot="1">
       <c r="A126" s="32">
         <v>607</v>
       </c>
@@ -25038,7 +25046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="127" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A127" s="31">
         <v>98</v>
       </c>
@@ -25066,7 +25074,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:13" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="128" spans="1:13" ht="19.2" customHeight="1" thickBot="1">
       <c r="A128" s="31">
         <v>99</v>
       </c>
@@ -25094,7 +25102,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="129" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="129" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A129" s="31">
         <v>100</v>
       </c>
@@ -25115,7 +25123,7 @@
       <c r="J129" s="22"/>
       <c r="K129" s="22"/>
     </row>
-    <row r="130" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="130" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A130" s="31">
         <v>101</v>
       </c>
@@ -25136,7 +25144,7 @@
       <c r="J130" s="22"/>
       <c r="K130" s="22"/>
     </row>
-    <row r="131" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="131" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A131" s="31">
         <v>102</v>
       </c>
@@ -25159,7 +25167,7 @@
       <c r="J131" s="22"/>
       <c r="K131" s="22"/>
     </row>
-    <row r="132" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="132" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A132" s="31">
         <v>106</v>
       </c>
@@ -25187,7 +25195,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="133" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="133" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A133" s="31">
         <v>107</v>
       </c>
@@ -25215,7 +25223,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="134" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="134" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A134" s="31">
         <v>103</v>
       </c>
@@ -25243,7 +25251,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="135" spans="1:12" ht="15.75" thickBot="1">
+    <row r="135" spans="1:12" ht="15" thickBot="1">
       <c r="B135" s="23" t="s">
         <v>479</v>
       </c>
@@ -25263,7 +25271,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="136" spans="1:12" ht="15.75" thickBot="1">
+    <row r="136" spans="1:12" ht="15" thickBot="1">
       <c r="B136" s="44" t="s">
         <v>480</v>
       </c>
@@ -25281,7 +25289,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="137" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="137" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A137" s="31">
         <v>108</v>
       </c>
@@ -25304,7 +25312,7 @@
       <c r="J137" s="22"/>
       <c r="K137" s="22"/>
     </row>
-    <row r="138" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="138" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A138" s="31">
         <v>109</v>
       </c>
@@ -25327,7 +25335,7 @@
       <c r="J138" s="22"/>
       <c r="K138" s="22"/>
     </row>
-    <row r="139" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="139" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A139" s="31">
         <v>110</v>
       </c>
@@ -25350,7 +25358,7 @@
       <c r="J139" s="22"/>
       <c r="K139" s="22"/>
     </row>
-    <row r="140" spans="1:12" ht="19.149999999999999" customHeight="1" thickBot="1">
+    <row r="140" spans="1:12" ht="19.2" customHeight="1" thickBot="1">
       <c r="A140" s="31">
         <v>111</v>
       </c>
@@ -25391,7 +25399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:12" ht="15.75" thickBot="1">
+    <row r="142" spans="1:12" ht="15" thickBot="1">
       <c r="B142" s="23" t="s">
         <v>563</v>
       </c>

</xml_diff>